<commit_message>
Reconcile all weekly deck assignments
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
+++ b/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rf3719c01aae4436a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="R17c424dd85414acd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="Rce8dee49d9eb4d8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R430e0f9c27c74f19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="R13a82c3c31174242"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="Ra5ff620ecdfa4dd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R3030208b8d9644ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="R30b31aa5c77b4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="R337fca7f276047c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R998a303668614c0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="R320c77bcd1c24532"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="Rd0a7cd389bb44bfc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -183,9 +183,6 @@
     <x:t xml:space="preserve">Weekly Focus</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Slide Deck(s)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Required Print Materials</x:t>
   </x:si>
   <x:si>
@@ -198,9 +195,6 @@
     <x:t xml:space="preserve">Implementation Notes</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 1: Authentic Research Course Launch; Deck 3: Research Ethics, Safety, and Integrity</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Launch reflection, identity inventory, ethics agreement, top five research areas</x:t>
   </x:si>
   <x:si>
@@ -210,9 +204,6 @@
     <x:t xml:space="preserve">No final project decisions yet; expand curiosity before narrowing</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 2: From Topic to Research Question; Deck 4: Experimental &amp; Engineering Design</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Experimental design practice, topic-to-question organizer, question quality test, preliminary pitch</x:t>
   </x:si>
   <x:si>
@@ -222,9 +213,6 @@
     <x:t xml:space="preserve">Students should leave with a promising direction, not a finalized plan</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 5: Building a Formal Research Plan</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Refined question, background notes, hypothesis/design criteria, evidence plan</x:t>
   </x:si>
   <x:si>
@@ -243,9 +231,6 @@
     <x:t xml:space="preserve">No testing begins until approval conditions are met</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 6: Pilot Testing; Deck 7: Research Journals and Documentation</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Pilot test plan, journal setup, first journal entries, safety check</x:t>
   </x:si>
   <x:si>
@@ -255,9 +240,6 @@
     <x:t xml:space="preserve">Students not approved continue planning revisions</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 8: Troubleshooting and Responsible Project Pivots</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Troubleshooting log, revision decision, brief progress update</x:t>
   </x:si>
   <x:si>
@@ -267,9 +249,6 @@
     <x:t xml:space="preserve">Do not let students drift into full data collection without a decision</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 8 revisit as needed</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Revised procedure, updated data table, peer procedure feedback, teacher approval checkpoint</x:t>
   </x:si>
   <x:si>
@@ -279,9 +258,6 @@
     <x:t xml:space="preserve">Vague data tables should trigger revision</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">No new core deck; use work-session slides as needed</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Formal data collection log, journal entries, first raw data checkpoint</x:t>
   </x:si>
   <x:si>
@@ -291,9 +267,6 @@
     <x:t xml:space="preserve">Students behind continue targeted revision or pilot testing</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">No new core deck; reference Deck 9 concepts if needed</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Updated raw data records, weekly check-in, data quality review</x:t>
   </x:si>
   <x:si>
@@ -303,9 +276,6 @@
     <x:t xml:space="preserve">Questionable data should be flagged, not deleted</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 8 revisit for project pivots</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Troubleshooting conference prep, mentor feedback log, documented revision or pivot</x:t>
   </x:si>
   <x:si>
@@ -315,9 +285,6 @@
     <x:t xml:space="preserve">A pivot requires evidence, documentation, and approval</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">No new core deck</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Updated raw data set, reliability/completeness check, updated timeline</x:t>
   </x:si>
   <x:si>
@@ -354,9 +321,6 @@
     <x:t xml:space="preserve">Last realistic week for major data collection in many calendars</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 9: Data Organization, Raw vs. Clean Data</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Organized raw data folder/spreadsheet, data audit checklist, missing-data plan</x:t>
   </x:si>
   <x:si>
@@ -366,9 +330,6 @@
     <x:t xml:space="preserve">Preserve raw data before cleaning</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 9 revisit</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Final journal check, readiness review, organized data set, unit reflection</x:t>
   </x:si>
   <x:si>
@@ -378,9 +339,6 @@
     <x:t xml:space="preserve">Students should leave knowing what can and cannot be analyzed</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 9: Data Organization; Deck 10: Choosing the Right Analysis Method</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Raw data inventory, clean data set, decision log, data audit</x:t>
   </x:si>
   <x:si>
@@ -390,9 +348,6 @@
     <x:t xml:space="preserve">Do not allow graphing before data are understandable</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 10: Choosing the Right Analysis Method</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Analysis plan, calculation/statistics notes, engineering performance analysis where applicable</x:t>
   </x:si>
   <x:si>
@@ -402,9 +357,6 @@
     <x:t xml:space="preserve">Advanced methods are only useful when they fit the question</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 11: Graphing and Visual Ethics; Deck 12: Error, Uncertainty, and Limitations</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Draft and final analysis visuals, captions, limitations review, gallery feedback</x:t>
   </x:si>
   <x:si>
@@ -414,9 +366,6 @@
     <x:t xml:space="preserve">Simple honest visuals beat flashy misleading ones</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 12 revisit as needed</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CER organizer, hypothesis/design review, interpretation notes, analysis summary, Unit 5 readiness</x:t>
   </x:si>
   <x:si>
@@ -426,18 +375,12 @@
     <x:t xml:space="preserve">Students need honest interpretation, not perfect results</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 13: Scientific Report Structure</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Annotated model report, strong/weak comparison, report planning map</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">This week is architecture, not polished writing</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 13 reference</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Introduction planning organizer, introduction draft, peer feedback</x:t>
   </x:si>
   <x:si>
@@ -456,18 +399,12 @@
     <x:t xml:space="preserve">Methods may reveal limitations to discuss later</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 11 reference for visual standards</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Final/near-final visuals, captions, results draft, graph critique feedback</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Not every graph belongs in the report</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 14: Writing the Discussion with CER</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CER organizer, limitations organizer, discussion draft, future work paragraph</x:t>
   </x:si>
   <x:si>
@@ -477,9 +414,6 @@
     <x:t xml:space="preserve">Students often overstate conclusions here</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 13 reference as needed</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Conclusion draft, complete Draft 1, self-assessment checklist, revision priorities</x:t>
   </x:si>
   <x:si>
@@ -489,18 +423,12 @@
     <x:t xml:space="preserve">Complete draft first, polish later</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 15: Peer Review and Scientific Revision</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Peer review forms, revision plan, revised Draft 2</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Conversation matters more than the form alone</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 16: Designing a Research Poster/Board; Deck 17 preview if needed</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Visual aid, speaking notes, practice feedback, presentation reflection</x:t>
   </x:si>
   <x:si>
@@ -510,9 +438,6 @@
     <x:t xml:space="preserve">Students should practice explaining, not reading</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 17: Oral Presentation Skills for Research</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Readiness check, research story refinement, revised speaking notes, three-length practice</x:t>
   </x:si>
   <x:si>
@@ -522,9 +447,6 @@
     <x:t xml:space="preserve">A presentation is not a spoken report</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 17 revisit</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Partner/small-group feedback, audience adaptation planner, revision log</x:t>
   </x:si>
   <x:si>
@@ -534,9 +456,6 @@
     <x:t xml:space="preserve">Confidence comes from repetition</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 18: Answering Questions Like a Scientist</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Q&amp;A guide, evidence defense organizer, mock Q&amp;A reflection, revised answers</x:t>
   </x:si>
   <x:si>
@@ -546,9 +465,6 @@
     <x:t xml:space="preserve">I don't know yet can be a scientific answer</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 16 and Deck 18 reference as needed</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Final product check, showcase readiness checklist, professionalism agreement, final rehearsal feedback</x:t>
   </x:si>
   <x:si>
@@ -558,9 +474,6 @@
     <x:t xml:space="preserve">Build in backup plans for tech and absences</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck 19: Final Reflection and Research Portfolio</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Final reflection, portfolio, optional next-step plan, course feedback/legacy reflection</x:t>
   </x:si>
   <x:si>
@@ -585,436 +498,367 @@
     <x:t xml:space="preserve">Primary Unit</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Best Week(s)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Instructional Purpose</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Authentic Research Course Launch</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Course launch and STARLAB identity</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">From Topic to Research Question</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Topic narrowing and question quality</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Research Ethics, Safety, and Integrity</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unit 1 / Unit 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Ethics, safety, and approval culture</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Experimental &amp; Engineering Design Basics</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Variables, controls, criteria, constraints</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Building a Formal Research Plan</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Formal research planning and approval</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Pilot Testing</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Testing small before full data collection</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Research Journals and Documentation</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Journal setup and scientific documentation</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Troubleshooting and Responsible Project Pivots</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Diagnose, revise, document, pivot responsibly</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Data Organization: Raw Data vs. Clean Data</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unit 3 / Unit 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Preserve raw data and create clean copies</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Choosing the Right Data Analysis Method</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Match data type to analysis method</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Graphing and Visual Ethics</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unit 4 / Unit 5</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clear, honest data visuals</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Error, Uncertainty, and Limitations</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Interpret evidence with caution</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Scientific Report Structure</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Report architecture and planning</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Writing the Discussion: CER</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Claim-evidence-reasoning, limitations, future work</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Peer Review and Scientific Revision</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Structured feedback and revision</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Designing a Research Poster or Presentation Board</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unit 5 / Unit 6</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Visual aid and showcase preparation</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Oral Presentation Skills for Research</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Research story, speaking notes, practice</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Answering Questions Like a Scientist</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Q&amp;A, evidence defense, scientific humility</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Final Reflection and Research Portfolio</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Portfolio, reflection, continuation planning</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unit Overview and Portal Placement</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Use this as the top-level map for the online portal</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unit Title</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Purpose</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Decks</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Major Products</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">STARLAB Major Checkpoints</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Teacher-facing milestones, approval gates, and course-wide decision points</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Timing</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Checkpoint</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Student Readiness Evidence</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Teacher Move</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Week 1</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">U1 H1, H2, H3; U1 Apps A-C</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Course launch and STARLAB identity</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">From Topic to Research Question</x:t>
+    <x:t xml:space="preserve">Course launch</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students understand STARLAB culture and research expectations</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Collect launch reflection and identity inventory</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Week 2</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Topic narrowing and question quality</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Research Ethics, Safety, and Integrity</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 1 / Unit 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 1 or Week 4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">U1 H4; U2 H9, H10; U2 Apps E, F, H</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ethics, safety, and approval culture</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Experimental &amp; Engineering Design Basics</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 2 or Week 3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Variables, controls, criteria, constraints</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Building a Formal Research Plan</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">U2 H1-H13; U2 App H</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Formal research planning and approval</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Pilot Testing</x:t>
+    <x:t xml:space="preserve">Preliminary project pitch</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students have at least one promising research direction</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Do not require final project decisions yet</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Formal research plan approval</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Week 5</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">U3 H1, H4, H5; U3 Apps A, C, E</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Testing small before full data collection</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Research Journals and Documentation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">U3 H2, H3, H4; U3 App B</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Journal setup and scientific documentation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Troubleshooting and Responsible Project Pivots</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weeks 6-10</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">U3 H4-H6, H11-H12; U3 Apps D, E, K</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Diagnose, revise, document, pivot responsibly</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Data Organization: Raw Data vs. Clean Data</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 / Unit 4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weeks 15-17</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">U4 H1-H4; U4 Apps A-C; optional U3 H17-H18</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Preserve raw data and create clean copies</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Choosing the Right Data Analysis Method</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weeks 17-18</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">U4 H5-H8; U4 Apps D-G</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Match data type to analysis method</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Graphing and Visual Ethics</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 4 / Unit 5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weeks 19 and 24</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Clear, honest data visuals</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Error, Uncertainty, and Limitations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weeks 19-20</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Interpret evidence with caution</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Scientific Report Structure</x:t>
+    <x:t xml:space="preserve">Pilot testing launch</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students test a small piece of their method or design</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Require journal setup and safety check</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 6-7</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Method revision gate</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Check revised procedures and data tables</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 8</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">First data checkpoint</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students show raw data and documentation</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 12</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Mid-project progress report</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students summarize completed work, preliminary evidence, challenges, and next steps</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Create recovery plans for students with limited data</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 16</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Readiness for analysis</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students have organized data and limitations identified</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Approve Unit 4 readiness categories</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 17</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clean data audit</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Raw data preserved and clean data copy created</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Stop analysis if data are not understandable</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 18</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Analysis plan checkpoint</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students choose calculations/statistics/metrics that fit their question</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Avoid unnecessary advanced methods</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 19</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Visual and limitations review</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Graphs/visuals are clear and honest; limitations are named</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Check labels, units, captions, error/uncertainty</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 20</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Unit 5 readiness</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students have interpretation notes and analysis summary</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Prevent overclaiming before report writing</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Week 21</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">U5 H1-H2; U5 Apps A, L</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Report architecture and planning</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Writing the Discussion: CER</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 25</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">U5 H6; U5 Apps H-I</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Claim-evidence-reasoning, limitations, future work</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Peer Review and Scientific Revision</x:t>
+    <x:t xml:space="preserve">Students map project evidence into report sections</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 26</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Complete Draft 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students submit a complete imperfect report draft</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Make revision possible</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Week 27</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">U5 H8-H9; U5 Apps M-N</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Structured feedback and revision</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Designing a Research Poster or Presentation Board</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 5 / Unit 6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weeks 28 and 32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visual aid and showcase preparation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Oral Presentation Skills for Research</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weeks 29-30</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Research story, speaking notes, practice</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Answering Questions Like a Scientist</x:t>
+    <x:t xml:space="preserve">Peer review and revision</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students complete structured peer review and revision plan</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Require specific, evidence-based feedback</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 28</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students have visual aid and practice presentation feedback</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Week 31</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">U6 H7-H9; U6 Apps F-H</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Q&amp;A, evidence defense, scientific humility</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Final Reflection and Research Portfolio</x:t>
+    <x:t xml:space="preserve">Q&amp;A readiness</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Students prepare evidence-based responses to likely questions</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Teach scientific humility and limitations language</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 32</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Showcase readiness</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Final visual product and logistics are ready</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Confirm backup plans and professionalism expectations</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Week 33</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Week 34</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Portfolio, reflection, continuation planning</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit Overview and Portal Placement</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Use this as the top-level map for the online portal</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit Title</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Purpose</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Decks</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Major Products</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">STARLAB Major Checkpoints</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Teacher-facing milestones, approval gates, and course-wide decision points</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Timing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Checkpoint</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Student Readiness Evidence</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Teacher Move</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Course launch</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students understand STARLAB culture and research expectations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Collect launch reflection and identity inventory</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Preliminary project pitch</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have at least one promising research direction</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Do not require final project decisions yet</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Formal research plan approval</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Pilot testing launch</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students test a small piece of their method or design</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Require journal setup and safety check</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 6-7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Method revision gate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Check revised procedures and data tables</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">First data checkpoint</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students show raw data and documentation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 12</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mid-project progress report</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students summarize completed work, preliminary evidence, challenges, and next steps</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Create recovery plans for students with limited data</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 16</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Readiness for analysis</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have organized data and limitations identified</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Approve Unit 4 readiness categories</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 17</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Clean data audit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Raw data preserved and clean data copy created</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Stop analysis if data are not understandable</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 18</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Analysis plan checkpoint</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students choose calculations/statistics/metrics that fit their question</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Avoid unnecessary advanced methods</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 19</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visual and limitations review</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Graphs/visuals are clear and honest; limitations are named</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Check labels, units, captions, error/uncertainty</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 20</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 5 readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have interpretation notes and analysis summary</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Prevent overclaiming before report writing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students map project evidence into report sections</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 26</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Complete Draft 1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students submit a complete imperfect report draft</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Make revision possible</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Peer review and revision</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students complete structured peer review and revision plan</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Require specific, evidence-based feedback</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 28</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have visual aid and practice presentation feedback</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Q&amp;A readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students prepare evidence-based responses to likely questions</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Teach scientific humility and limitations language</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Showcase readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Final visual product and logistics are ready</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Confirm backup plans and professionalism expectations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 33</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Portfolio and reflection</x:t>
@@ -1133,7 +977,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -1178,6 +1022,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -3471,7 +3321,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c71d8228d414e3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26f1583fba4047bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3516,7 +3366,7 @@
       <x:c r="I4" s="4"/>
       <x:c r="J4" s="4"/>
     </x:row>
-    <x:row r="5" ht="31.5" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="s">
         <x:v>53</x:v>
       </x:c>
@@ -3529,26 +3379,26 @@
       <x:c r="D5" s="6" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="E5" s="6" t="s">
+      <x:c r="E5" s="15" t="str">
+        <x:v>Deck Use</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="F5" s="6" t="s">
+      <x:c r="G5" s="6" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="G5" s="6" t="s">
+      <x:c r="H5" s="6" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="H5" s="6" t="s">
+      <x:c r="I5" s="6" t="s">
         <x:v>59</x:v>
-      </x:c>
-      <x:c r="I5" s="6" t="s">
-        <x:v>60</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
         <x:v>Optional / Teacher Reference</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="36" hidden="0" customHeight="1">
       <x:c r="A6" s="7">
         <x:v>1.0</x:v>
       </x:c>
@@ -3559,24 +3409,24 @@
       <x:c r="D6" s="7" t="str">
         <x:v>Course launch, research culture, curiosity, and ethics</x:v>
       </x:c>
-      <x:c r="E6" s="7" t="s">
-        <x:v>61</x:v>
+      <x:c r="E6" s="16" t="str">
+        <x:v>Primary - Deck 1: Authentic Research Course Launch; Deck 3: Research Ethics, Safety, and Integrity</x:v>
       </x:c>
       <x:c r="F6" s="7" t="str">
         <x:v>U1 H1; U1 H2; U1 H3; U1 H4; U1 App A; U1 App B; U1 App C</x:v>
       </x:c>
       <x:c r="G6" s="7" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H6" s="7" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="H6" s="7" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="I6" s="7" t="s">
-        <x:v>64</x:v>
-      </x:c>
       <x:c r="J6" s="13" t="str"/>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="7">
         <x:v>2.0</x:v>
       </x:c>
@@ -3587,26 +3437,26 @@
       <x:c r="D7" s="7" t="str">
         <x:v>Experimental design, feasibility, and preliminary research questions</x:v>
       </x:c>
-      <x:c r="E7" s="7" t="s">
-        <x:v>65</x:v>
+      <x:c r="E7" s="16" t="str">
+        <x:v>Primary - Deck 2: From Topic to Research Question; Deck 4: Experimental &amp; Engineering Design</x:v>
       </x:c>
       <x:c r="F7" s="7" t="str">
         <x:v>U1 H5; U1 H6; U1 H7; U1 H8; U1 App D; U1 App E; U1 App F; U1 App G; U1 App H</x:v>
       </x:c>
       <x:c r="G7" s="7" t="s">
-        <x:v>66</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H7" s="7" t="s">
-        <x:v>67</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="I7" s="7" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="J7" s="14" t="str">
         <x:v>U1 App I</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="36" hidden="0" customHeight="1">
       <x:c r="A8" s="7">
         <x:v>3.0</x:v>
       </x:c>
@@ -3617,24 +3467,24 @@
       <x:c r="D8" s="7" t="str">
         <x:v>From project idea to testable plan</x:v>
       </x:c>
-      <x:c r="E8" s="7" t="s">
-        <x:v>69</x:v>
+      <x:c r="E8" s="16" t="str">
+        <x:v>Primary - Deck 5: Building a Formal Research Plan; Revisit / Reference - Deck 4: Experimental &amp; Engineering Design</x:v>
       </x:c>
       <x:c r="F8" s="7" t="str">
         <x:v>U2 H1; U2 H2; U2 H3; U2 H4; U2 H5; U2 App A; U2 App B; U2 App C; U2 App D</x:v>
       </x:c>
       <x:c r="G8" s="7" t="s">
-        <x:v>70</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="H8" s="7" t="s">
-        <x:v>71</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="I8" s="7" t="s">
-        <x:v>72</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="J8" s="13" t="str"/>
     </x:row>
-    <x:row r="9" ht="34" customHeight="1">
+    <x:row r="9" ht="36" hidden="0" customHeight="1">
       <x:c r="A9" s="7">
         <x:v>4.0</x:v>
       </x:c>
@@ -3645,26 +3495,26 @@
       <x:c r="D9" s="7" t="str">
         <x:v>Formal research plan, safety, ethics, and approval</x:v>
       </x:c>
-      <x:c r="E9" s="7" t="s">
-        <x:v>69</x:v>
+      <x:c r="E9" s="16" t="str">
+        <x:v>Primary - Deck 5: Building a Formal Research Plan; Revisit / Reference - Deck 3: Research Ethics, Safety, and Integrity</x:v>
       </x:c>
       <x:c r="F9" s="7" t="str">
         <x:v>U2 H6; U2 H7; U2 H8; U2 H9; U2 H10; U2 H11; U2 H12; U2 H13; U2 App E; U2 App F; U2 App G; U2 App H</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
-        <x:v>73</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="H9" s="7" t="s">
-        <x:v>74</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I9" s="7" t="s">
-        <x:v>75</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str">
         <x:v>U2 AppI; U2 AppJ; district-supplied approval and safety forms as applicable</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="24" hidden="0" customHeight="1">
       <x:c r="A10" s="7">
         <x:v>5.0</x:v>
       </x:c>
@@ -3675,24 +3525,24 @@
       <x:c r="D10" s="7" t="str">
         <x:v>Launching pilot testing and research journals</x:v>
       </x:c>
-      <x:c r="E10" s="7" t="s">
-        <x:v>76</x:v>
+      <x:c r="E10" s="16" t="str">
+        <x:v>Primary - Deck 6: Pilot Testing; Deck 7: Research Journals and Documentation</x:v>
       </x:c>
       <x:c r="F10" s="7" t="str">
         <x:v>U3 H1; U3 H2; U3 H3; U3 App A; U3 App B; U3 App C</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>77</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H10" s="7" t="s">
-        <x:v>78</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="I10" s="7" t="s">
-        <x:v>79</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="J10" s="13" t="str"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="7">
         <x:v>6.0</x:v>
       </x:c>
@@ -3703,24 +3553,24 @@
       <x:c r="D11" s="7" t="str">
         <x:v>Pilot testing, observation, and troubleshooting</x:v>
       </x:c>
-      <x:c r="E11" s="7" t="s">
-        <x:v>80</x:v>
+      <x:c r="E11" s="16" t="str">
+        <x:v>Primary - Deck 8: Troubleshooting and Responsible Project Pivots</x:v>
       </x:c>
       <x:c r="F11" s="7" t="str">
         <x:v>U3 H4; U3 H5; U3 App D; U3 App E</x:v>
       </x:c>
       <x:c r="G11" s="7" t="s">
-        <x:v>81</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H11" s="7" t="s">
-        <x:v>82</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="I11" s="7" t="s">
-        <x:v>83</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="J11" s="14" t="str"/>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="7">
         <x:v>7.0</x:v>
       </x:c>
@@ -3731,24 +3581,24 @@
       <x:c r="D12" s="7" t="str">
         <x:v>Revising methods and data collection tools</x:v>
       </x:c>
-      <x:c r="E12" s="7" t="s">
-        <x:v>84</x:v>
+      <x:c r="E12" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 8</x:v>
       </x:c>
       <x:c r="F12" s="7" t="str">
         <x:v>U3 H6; U3 H7; U3 App F; U3 App G</x:v>
       </x:c>
       <x:c r="G12" s="7" t="s">
-        <x:v>85</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H12" s="7" t="s">
-        <x:v>86</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="I12" s="7" t="s">
-        <x:v>87</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J12" s="13" t="str"/>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="7">
         <x:v>8.0</x:v>
       </x:c>
@@ -3759,26 +3609,26 @@
       <x:c r="D13" s="7" t="str">
         <x:v>Beginning systematic data collection</x:v>
       </x:c>
-      <x:c r="E13" s="7" t="s">
-        <x:v>88</x:v>
+      <x:c r="E13" s="16" t="str">
+        <x:v>No New Deck - systematic data collection work sessions</x:v>
       </x:c>
       <x:c r="F13" s="7" t="str">
         <x:v>U3 H8; U3 H9; U3 App H</x:v>
       </x:c>
       <x:c r="G13" s="7" t="s">
-        <x:v>89</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="H13" s="7" t="s">
-        <x:v>90</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="I13" s="7" t="s">
-        <x:v>91</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str">
         <x:v>U3 App I</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="7">
         <x:v>9.0</x:v>
       </x:c>
@@ -3789,26 +3639,26 @@
       <x:c r="D14" s="7" t="str">
         <x:v>Continuing data collection and monitoring quality</x:v>
       </x:c>
-      <x:c r="E14" s="7" t="s">
-        <x:v>92</x:v>
+      <x:c r="E14" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 9 as needed</x:v>
       </x:c>
       <x:c r="F14" s="7" t="str">
         <x:v>U3 H9; U3 H10</x:v>
       </x:c>
       <x:c r="G14" s="7" t="s">
-        <x:v>93</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="H14" s="7" t="s">
-        <x:v>94</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="I14" s="7" t="s">
-        <x:v>95</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="J14" s="13" t="str">
         <x:v>U3 App J</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="7">
         <x:v>10.0</x:v>
       </x:c>
@@ -3819,26 +3669,26 @@
       <x:c r="D15" s="7" t="str">
         <x:v>Troubleshooting, iteration, and mentor feedback</x:v>
       </x:c>
-      <x:c r="E15" s="7" t="s">
-        <x:v>96</x:v>
+      <x:c r="E15" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 8</x:v>
       </x:c>
       <x:c r="F15" s="7" t="str">
         <x:v>U3 H11; U3 H12</x:v>
       </x:c>
       <x:c r="G15" s="7" t="s">
-        <x:v>97</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="H15" s="7" t="s">
-        <x:v>98</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="I15" s="7" t="s">
-        <x:v>99</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="J15" s="14" t="str">
         <x:v>U3 App K; U3 App L</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="7">
         <x:v>11.0</x:v>
       </x:c>
@@ -3849,26 +3699,26 @@
       <x:c r="D16" s="7" t="str">
         <x:v>Expanding trials and checking reliability</x:v>
       </x:c>
-      <x:c r="E16" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="E16" s="16" t="str">
+        <x:v>No New Deck - data collection and reliability work sessions</x:v>
       </x:c>
       <x:c r="F16" s="7" t="str">
         <x:v>U3 H9; U3 H13</x:v>
       </x:c>
       <x:c r="G16" s="7" t="s">
-        <x:v>101</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="H16" s="7" t="s">
-        <x:v>102</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="I16" s="7" t="s">
-        <x:v>103</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="J16" s="13" t="str">
         <x:v>U3 App M</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="7">
         <x:v>12.0</x:v>
       </x:c>
@@ -3879,26 +3729,26 @@
       <x:c r="D17" s="7" t="str">
         <x:v>Midpoint review and progress reporting</x:v>
       </x:c>
-      <x:c r="E17" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="E17" s="16" t="str">
+        <x:v>No New Deck - midpoint review and progress reporting</x:v>
       </x:c>
       <x:c r="F17" s="7" t="str">
         <x:v>U3 H14; U3 App N</x:v>
       </x:c>
       <x:c r="G17" s="7" t="s">
-        <x:v>104</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="H17" s="7" t="s">
-        <x:v>105</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="I17" s="7" t="s">
-        <x:v>106</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="J17" s="14" t="str">
         <x:v>U3 App O</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="24" hidden="0" customHeight="1">
       <x:c r="A18" s="7">
         <x:v>13.0</x:v>
       </x:c>
@@ -3909,26 +3759,26 @@
       <x:c r="D18" s="7" t="str">
         <x:v>Continued data collection after feedback</x:v>
       </x:c>
-      <x:c r="E18" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="E18" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 8 as needed</x:v>
       </x:c>
       <x:c r="F18" s="7" t="str">
         <x:v>U3 H9; U3 H15</x:v>
       </x:c>
       <x:c r="G18" s="7" t="s">
-        <x:v>107</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H18" s="7" t="s">
-        <x:v>108</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="I18" s="7" t="s">
-        <x:v>109</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="J18" s="13" t="str">
         <x:v>U3 App P</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="24" hidden="0" customHeight="1">
       <x:c r="A19" s="7">
         <x:v>14.0</x:v>
       </x:c>
@@ -3939,24 +3789,24 @@
       <x:c r="D19" s="7" t="str">
         <x:v>Completing major trials or prototype iterations</x:v>
       </x:c>
-      <x:c r="E19" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="E19" s="16" t="str">
+        <x:v>No New Deck - major trial or prototype completion work sessions</x:v>
       </x:c>
       <x:c r="F19" s="7" t="str">
         <x:v>U3 H9; U3 H16</x:v>
       </x:c>
       <x:c r="G19" s="7" t="s">
-        <x:v>110</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="H19" s="7" t="s">
-        <x:v>111</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I19" s="7" t="s">
-        <x:v>112</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="J19" s="14" t="str"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="7">
         <x:v>15.0</x:v>
       </x:c>
@@ -3967,24 +3817,24 @@
       <x:c r="D20" s="7" t="str">
         <x:v>Data organization and completeness audit</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="s">
-        <x:v>113</x:v>
+      <x:c r="E20" s="16" t="str">
+        <x:v>Primary - Deck 9: Data Organization, Raw vs. Clean Data</x:v>
       </x:c>
       <x:c r="F20" s="7" t="str">
         <x:v>U3 H17; U3 App Q; U3 App R</x:v>
       </x:c>
       <x:c r="G20" s="7" t="s">
-        <x:v>114</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="H20" s="7" t="s">
-        <x:v>115</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="I20" s="7" t="s">
-        <x:v>116</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="J20" s="13" t="str"/>
     </x:row>
-    <x:row r="21" ht="15.75" customHeight="1">
+    <x:row r="21" ht="24" hidden="0" customHeight="1">
       <x:c r="A21" s="7">
         <x:v>16.0</x:v>
       </x:c>
@@ -3995,26 +3845,26 @@
       <x:c r="D21" s="7" t="str">
         <x:v>Unit 3 closure and readiness for analysis</x:v>
       </x:c>
-      <x:c r="E21" s="7" t="s">
-        <x:v>117</x:v>
+      <x:c r="E21" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 9</x:v>
       </x:c>
       <x:c r="F21" s="7" t="str">
         <x:v>U3 H18; U3 H19</x:v>
       </x:c>
       <x:c r="G21" s="7" t="s">
-        <x:v>118</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="H21" s="7" t="s">
-        <x:v>119</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="I21" s="7" t="s">
-        <x:v>120</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="J21" s="14" t="str">
         <x:v>U3 App S; U3 App T; U3 App U</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15.75" customHeight="1">
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
       <x:c r="A22" s="7">
         <x:v>17.0</x:v>
       </x:c>
@@ -4025,24 +3875,24 @@
       <x:c r="D22" s="7" t="str">
         <x:v>Data organization, cleaning, and audit</x:v>
       </x:c>
-      <x:c r="E22" s="7" t="s">
-        <x:v>121</x:v>
+      <x:c r="E22" s="16" t="str">
+        <x:v>Primary - Deck 9: Data Organization; Deck 10: Choosing the Right Analysis Method</x:v>
       </x:c>
       <x:c r="F22" s="7" t="str">
         <x:v>U4 H1; U4 H2; U4 H3; U4 H4; U4 App A; U4 App B; U4 App C</x:v>
       </x:c>
       <x:c r="G22" s="7" t="s">
-        <x:v>122</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="H22" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="I22" s="7" t="s">
-        <x:v>124</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="J22" s="13" t="str"/>
     </x:row>
-    <x:row r="23" ht="15.75" customHeight="1">
+    <x:row r="23" ht="24" hidden="0" customHeight="1">
       <x:c r="A23" s="7">
         <x:v>18.0</x:v>
       </x:c>
@@ -4053,24 +3903,24 @@
       <x:c r="D23" s="7" t="str">
         <x:v>Calculations, statistics, and analysis methods</x:v>
       </x:c>
-      <x:c r="E23" s="7" t="s">
-        <x:v>125</x:v>
+      <x:c r="E23" s="16" t="str">
+        <x:v>Primary - Deck 10: Choosing the Right Analysis Method</x:v>
       </x:c>
       <x:c r="F23" s="7" t="str">
         <x:v>U4 H5; U4 H6; U4 H7; U4 H8; U4 App D; U4 App E; U4 App F; U4 App G</x:v>
       </x:c>
       <x:c r="G23" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="H23" s="7" t="s">
-        <x:v>127</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="I23" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="J23" s="14" t="str"/>
     </x:row>
-    <x:row r="24" ht="15.75" customHeight="1">
+    <x:row r="24" ht="24" hidden="0" customHeight="1">
       <x:c r="A24" s="7">
         <x:v>19.0</x:v>
       </x:c>
@@ -4081,24 +3931,24 @@
       <x:c r="D24" s="7" t="str">
         <x:v>Graphs, tables, visuals, error, and uncertainty</x:v>
       </x:c>
-      <x:c r="E24" s="7" t="s">
-        <x:v>129</x:v>
+      <x:c r="E24" s="16" t="str">
+        <x:v>Primary - Deck 11: Graphing and Visual Ethics; Deck 12: Error, Uncertainty, and Limitations</x:v>
       </x:c>
       <x:c r="F24" s="7" t="str">
         <x:v>U4 H9; U4 H10; U4 H11; U4 H12; U4 App H; U4 App I; U4 App J; U4 App K</x:v>
       </x:c>
       <x:c r="G24" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="H24" s="7" t="s">
-        <x:v>131</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="I24" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="J24" s="13" t="str"/>
     </x:row>
-    <x:row r="25" ht="34" customHeight="1">
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="7">
         <x:v>20.0</x:v>
       </x:c>
@@ -4109,26 +3959,26 @@
       <x:c r="D25" s="7" t="str">
         <x:v>Interpretation, claims, and transition to reporting</x:v>
       </x:c>
-      <x:c r="E25" s="7" t="s">
-        <x:v>133</x:v>
+      <x:c r="E25" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 12</x:v>
       </x:c>
       <x:c r="F25" s="7" t="str">
         <x:v>U4 H13; U4 H14; U4 H15; U4 H16; U4 H17; U4 App N</x:v>
       </x:c>
       <x:c r="G25" s="7" t="s">
-        <x:v>134</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="H25" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="I25" s="7" t="s">
-        <x:v>136</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="J25" s="14" t="str">
         <x:v>U4 App L; U4 App M; U4 App O; U4 App P; U4 App Q</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="15.75" customHeight="1">
+    <x:row r="26" ht="36" hidden="0" customHeight="1">
       <x:c r="A26" s="7">
         <x:v>21.0</x:v>
       </x:c>
@@ -4139,24 +3989,24 @@
       <x:c r="D26" s="7" t="str">
         <x:v>Understanding scientific reports</x:v>
       </x:c>
-      <x:c r="E26" s="7" t="s">
-        <x:v>137</x:v>
+      <x:c r="E26" s="16" t="str">
+        <x:v>Primary - Deck 13: Scientific Report Structure</x:v>
       </x:c>
       <x:c r="F26" s="7" t="str">
         <x:v>U5 H1; U5 H2; U5 App A; U5 App L</x:v>
       </x:c>
       <x:c r="G26" s="7" t="s">
-        <x:v>138</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="H26" s="7" t="str">
         <x:v>Shift students into scientific structure; set or confirm public showcase format, date, audience, and space six to eight weeks ahead</x:v>
       </x:c>
       <x:c r="I26" s="7" t="s">
-        <x:v>139</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="J26" s="13" t="str"/>
     </x:row>
-    <x:row r="27" ht="15.75" customHeight="1">
+    <x:row r="27" ht="24" hidden="0" customHeight="1">
       <x:c r="A27" s="7">
         <x:v>22.0</x:v>
       </x:c>
@@ -4167,24 +4017,24 @@
       <x:c r="D27" s="7" t="str">
         <x:v>Writing the introduction</x:v>
       </x:c>
-      <x:c r="E27" s="7" t="s">
-        <x:v>140</x:v>
+      <x:c r="E27" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 13</x:v>
       </x:c>
       <x:c r="F27" s="7" t="str">
         <x:v>U5 H3; U5 App B; U5 App C</x:v>
       </x:c>
       <x:c r="G27" s="7" t="s">
-        <x:v>141</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H27" s="7" t="s">
-        <x:v>142</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="I27" s="7" t="s">
-        <x:v>143</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="J27" s="14" t="str"/>
     </x:row>
-    <x:row r="28" ht="15.75" customHeight="1">
+    <x:row r="28" ht="24" hidden="0" customHeight="1">
       <x:c r="A28" s="7">
         <x:v>23.0</x:v>
       </x:c>
@@ -4195,24 +4045,24 @@
       <x:c r="D28" s="7" t="str">
         <x:v>Writing the methods section</x:v>
       </x:c>
-      <x:c r="E28" s="7" t="s">
-        <x:v>140</x:v>
+      <x:c r="E28" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 13</x:v>
       </x:c>
       <x:c r="F28" s="7" t="str">
         <x:v>U5 H4; U5 App D; U5 App E</x:v>
       </x:c>
       <x:c r="G28" s="7" t="s">
-        <x:v>144</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="H28" s="7" t="s">
-        <x:v>145</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="I28" s="7" t="s">
-        <x:v>146</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="J28" s="13" t="str"/>
     </x:row>
-    <x:row r="29" ht="15.75" customHeight="1">
+    <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="7">
         <x:v>24.0</x:v>
       </x:c>
@@ -4223,24 +4073,24 @@
       <x:c r="D29" s="7" t="str">
         <x:v>Results, figures, tables, and captions</x:v>
       </x:c>
-      <x:c r="E29" s="7" t="s">
-        <x:v>147</x:v>
+      <x:c r="E29" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 11</x:v>
       </x:c>
       <x:c r="F29" s="7" t="str">
         <x:v>U5 H5; U5 App F; U5 App G</x:v>
       </x:c>
       <x:c r="G29" s="7" t="s">
-        <x:v>148</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
         <x:v>Separate results from discussion; send invitations or confirm the public audience and district communication plan</x:v>
       </x:c>
       <x:c r="I29" s="7" t="s">
-        <x:v>149</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="J29" s="14" t="str"/>
     </x:row>
-    <x:row r="30" ht="15.75" customHeight="1">
+    <x:row r="30" ht="24" hidden="0" customHeight="1">
       <x:c r="A30" s="7">
         <x:v>25.0</x:v>
       </x:c>
@@ -4251,24 +4101,24 @@
       <x:c r="D30" s="7" t="str">
         <x:v>Writing the discussion</x:v>
       </x:c>
-      <x:c r="E30" s="7" t="s">
-        <x:v>150</x:v>
+      <x:c r="E30" s="16" t="str">
+        <x:v>Primary - Deck 14: Writing the Discussion with CER</x:v>
       </x:c>
       <x:c r="F30" s="7" t="str">
         <x:v>U5 H6; U5 App H; U5 App I</x:v>
       </x:c>
       <x:c r="G30" s="7" t="s">
-        <x:v>151</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="H30" s="7" t="s">
-        <x:v>152</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="I30" s="7" t="s">
-        <x:v>153</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="J30" s="13" t="str"/>
     </x:row>
-    <x:row r="31" ht="15.75" customHeight="1">
+    <x:row r="31" ht="24" hidden="0" customHeight="1">
       <x:c r="A31" s="7">
         <x:v>26.0</x:v>
       </x:c>
@@ -4279,24 +4129,24 @@
       <x:c r="D31" s="7" t="str">
         <x:v>Conclusion and full report assembly</x:v>
       </x:c>
-      <x:c r="E31" s="7" t="s">
-        <x:v>154</x:v>
+      <x:c r="E31" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 13</x:v>
       </x:c>
       <x:c r="F31" s="7" t="str">
         <x:v>U5 H7; U5 App J; U5 App K; U5 App L</x:v>
       </x:c>
       <x:c r="G31" s="7" t="s">
-        <x:v>155</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="H31" s="7" t="s">
-        <x:v>156</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="I31" s="7" t="s">
-        <x:v>157</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="J31" s="14" t="str"/>
     </x:row>
-    <x:row r="32" ht="15.75" customHeight="1">
+    <x:row r="32" ht="24" hidden="0" customHeight="1">
       <x:c r="A32" s="7">
         <x:v>27.0</x:v>
       </x:c>
@@ -4307,24 +4157,24 @@
       <x:c r="D32" s="7" t="str">
         <x:v>Peer review and revision</x:v>
       </x:c>
-      <x:c r="E32" s="7" t="s">
-        <x:v>158</x:v>
+      <x:c r="E32" s="16" t="str">
+        <x:v>Primary - Deck 15: Peer Review and Scientific Revision</x:v>
       </x:c>
       <x:c r="F32" s="7" t="str">
         <x:v>U5 H8; U5 H9; U5 App M; U5 App N</x:v>
       </x:c>
       <x:c r="G32" s="7" t="s">
-        <x:v>159</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="H32" s="7" t="str">
         <x:v>Structure specific peer feedback; finalize public event logistics, technology, accessibility, and assessment workflow</x:v>
       </x:c>
       <x:c r="I32" s="7" t="s">
-        <x:v>160</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="J32" s="13" t="str"/>
     </x:row>
-    <x:row r="33" ht="15.75" customHeight="1">
+    <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="7">
         <x:v>28.0</x:v>
       </x:c>
@@ -4335,26 +4185,26 @@
       <x:c r="D33" s="7" t="str">
         <x:v>Presentation design and practice</x:v>
       </x:c>
-      <x:c r="E33" s="7" t="s">
-        <x:v>161</x:v>
+      <x:c r="E33" s="16" t="str">
+        <x:v>Primary - Deck 16: Designing a Research Poster/Board; Preview / Reference - Deck 17</x:v>
       </x:c>
       <x:c r="F33" s="7" t="str">
         <x:v>U5 H10; U5 H11; U5 App O</x:v>
       </x:c>
       <x:c r="G33" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="H33" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="I33" s="7" t="s">
-        <x:v>164</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="J33" s="14" t="str">
         <x:v>U5 App Q</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="15.75" customHeight="1">
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
       <x:c r="A34" s="7">
         <x:v>29.0</x:v>
       </x:c>
@@ -4365,24 +4215,24 @@
       <x:c r="D34" s="7" t="str">
         <x:v>Final presentation readiness and message refinement</x:v>
       </x:c>
-      <x:c r="E34" s="7" t="s">
-        <x:v>165</x:v>
+      <x:c r="E34" s="16" t="str">
+        <x:v>Primary - Deck 17: Oral Presentation Skills for Research</x:v>
       </x:c>
       <x:c r="F34" s="7" t="str">
         <x:v>U6 H1; U6 H2; U6 H3; U6 App A; U6 App B; U6 App C</x:v>
       </x:c>
       <x:c r="G34" s="7" t="s">
-        <x:v>166</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="H34" s="7" t="s">
-        <x:v>167</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="I34" s="7" t="s">
-        <x:v>168</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="J34" s="13" t="str"/>
     </x:row>
-    <x:row r="35" ht="15.75" customHeight="1">
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
       <x:c r="A35" s="7">
         <x:v>30.0</x:v>
       </x:c>
@@ -4393,24 +4243,24 @@
       <x:c r="D35" s="7" t="str">
         <x:v>Practice presentations and audience adaptation</x:v>
       </x:c>
-      <x:c r="E35" s="7" t="s">
-        <x:v>169</x:v>
+      <x:c r="E35" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 17</x:v>
       </x:c>
       <x:c r="F35" s="7" t="str">
         <x:v>U6 H4; U6 H5; U6 H6; U6 App D; U6 App E</x:v>
       </x:c>
       <x:c r="G35" s="7" t="s">
-        <x:v>170</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="H35" s="7" t="s">
-        <x:v>171</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="I35" s="7" t="s">
-        <x:v>172</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="J35" s="14" t="str"/>
     </x:row>
-    <x:row r="36" ht="15.75" customHeight="1">
+    <x:row r="36" ht="24" hidden="0" customHeight="1">
       <x:c r="A36" s="7">
         <x:v>31.0</x:v>
       </x:c>
@@ -4421,24 +4271,24 @@
       <x:c r="D36" s="7" t="str">
         <x:v>Q&amp;A preparation and defense of evidence</x:v>
       </x:c>
-      <x:c r="E36" s="7" t="s">
-        <x:v>173</x:v>
+      <x:c r="E36" s="16" t="str">
+        <x:v>Primary - Deck 18: Answering Questions Like a Scientist</x:v>
       </x:c>
       <x:c r="F36" s="7" t="str">
         <x:v>U6 H7; U6 H8; U6 H9; U6 App F; U6 App G; U6 App H</x:v>
       </x:c>
       <x:c r="G36" s="7" t="s">
-        <x:v>174</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="H36" s="7" t="s">
-        <x:v>175</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="I36" s="7" t="s">
-        <x:v>176</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="J36" s="13" t="str"/>
     </x:row>
-    <x:row r="37" ht="15.75" customHeight="1">
+    <x:row r="37" ht="24" hidden="0" customHeight="1">
       <x:c r="A37" s="7">
         <x:v>32.0</x:v>
       </x:c>
@@ -4449,26 +4299,26 @@
       <x:c r="D37" s="7" t="str">
         <x:v>Final showcase preparation</x:v>
       </x:c>
-      <x:c r="E37" s="7" t="s">
-        <x:v>177</x:v>
+      <x:c r="E37" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Decks 16 and 18</x:v>
       </x:c>
       <x:c r="F37" s="7" t="str">
         <x:v>U6 H10; U6 H11; U6 H12</x:v>
       </x:c>
       <x:c r="G37" s="7" t="s">
-        <x:v>178</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="H37" s="7" t="s">
-        <x:v>179</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="I37" s="7" t="s">
-        <x:v>180</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="J37" s="14" t="str">
         <x:v>U6 App I; U6 App J; U6 App K</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="15.75" customHeight="1">
+    <x:row r="38" ht="36" hidden="0" customHeight="1">
       <x:c r="A38" s="7">
         <x:v>33.0</x:v>
       </x:c>
@@ -4479,8 +4329,8 @@
       <x:c r="D38" s="7" t="str">
         <x:v>Required public presentation or showcase</x:v>
       </x:c>
-      <x:c r="E38" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="E38" s="16" t="str">
+        <x:v>No New Deck - required public presentation or showcase</x:v>
       </x:c>
       <x:c r="F38" s="7" t="str">
         <x:v>U6 H13; U6 H14; U6 App L; U6 App M</x:v>
@@ -4498,7 +4348,7 @@
         <x:v>U6 App N</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="34" customHeight="1">
+    <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A39" s="7">
         <x:v>34.0</x:v>
       </x:c>
@@ -4509,20 +4359,20 @@
       <x:c r="D39" s="7" t="str">
         <x:v>Final reflection, portfolio, and next steps</x:v>
       </x:c>
-      <x:c r="E39" s="7" t="s">
-        <x:v>181</x:v>
+      <x:c r="E39" s="16" t="str">
+        <x:v>Primary - Deck 19: Final Reflection and Research Portfolio</x:v>
       </x:c>
       <x:c r="F39" s="7" t="str">
         <x:v>U6 H15; U6 H16; U6 H18</x:v>
       </x:c>
       <x:c r="G39" s="7" t="s">
-        <x:v>182</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="H39" s="7" t="s">
-        <x:v>183</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="I39" s="7" t="s">
-        <x:v>184</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="J39" s="14" t="str">
         <x:v>U6 H17; U6 App O; U6 App P; U6 App Q; U6 App R; U6 App S</x:v>
@@ -5953,7 +5803,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0ed4914e7654231"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34cebcbc746c4c61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5972,12 +5822,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>185</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>186</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -5995,480 +5845,480 @@
       <x:c r="I4" s="4"/>
       <x:c r="J4" s="4"/>
     </x:row>
-    <x:row r="5" ht="31.5" customHeight="1">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>187</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="s">
-        <x:v>190</x:v>
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="D5" s="15" t="str">
+        <x:v>Authoritative Week Use</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="F5" s="6" t="s">
-        <x:v>191</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
       <x:c r="I5" s="4"/>
       <x:c r="J5" s="4"/>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="7">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>192</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="s">
-        <x:v>193</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="s">
-        <x:v>194</x:v>
+      <x:c r="D6" s="16" t="str">
+        <x:v>Primary - Week 1</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="str">
+        <x:v>Week 1: U1 H1-H4; U1 Apps A-C</x:v>
       </x:c>
       <x:c r="F6" s="7" t="s">
-        <x:v>195</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="G6" s="4"/>
       <x:c r="H6" s="4"/>
       <x:c r="I6" s="4"/>
       <x:c r="J6" s="4"/>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="7">
         <x:v>2.0</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
-        <x:v>196</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="C7" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="D7" s="7" t="s">
-        <x:v>197</x:v>
+      <x:c r="D7" s="16" t="str">
+        <x:v>Primary - Week 2</x:v>
       </x:c>
       <x:c r="E7" s="7" t="str">
-        <x:v>U1 H3, H6-H8; U1 Apps E, G</x:v>
+        <x:v>Week 2: U1 H5-H8; U1 Apps D-H</x:v>
       </x:c>
       <x:c r="F7" s="7" t="s">
-        <x:v>198</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="G7" s="4"/>
       <x:c r="H7" s="4"/>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="24" hidden="0" customHeight="1">
       <x:c r="A8" s="7">
         <x:v>3.0</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
-        <x:v>199</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="D8" s="7" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="E8" s="7" t="s">
-        <x:v>202</x:v>
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>Primary - Week 1; Revisit / Reference - Week 4</x:v>
+      </x:c>
+      <x:c r="E8" s="7" t="str">
+        <x:v>Week 1: U1 H1-H4; U1 Apps A-C; Week 4: U2 H6-H13; U2 Apps E-H</x:v>
       </x:c>
       <x:c r="F8" s="7" t="s">
-        <x:v>203</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="G8" s="4"/>
       <x:c r="H8" s="4"/>
       <x:c r="I8" s="4"/>
       <x:c r="J8" s="4"/>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="24" hidden="0" customHeight="1">
       <x:c r="A9" s="7">
         <x:v>4.0</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
-        <x:v>204</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="D9" s="7" t="s">
-        <x:v>205</x:v>
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>Primary - Week 2; Revisit / Reference - Week 3</x:v>
       </x:c>
       <x:c r="E9" s="7" t="str">
-        <x:v>U1 H5; U1 Apps D, G; U2 H3-H5</x:v>
+        <x:v>Week 2: U1 H5-H8; U1 Apps D-H; Week 3: U2 H1-H5; U2 Apps A-D</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
-        <x:v>206</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="G9" s="4"/>
       <x:c r="H9" s="4"/>
       <x:c r="I9" s="4"/>
       <x:c r="J9" s="4"/>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="7">
         <x:v>5.0</x:v>
       </x:c>
       <x:c r="B10" s="7" t="s">
-        <x:v>207</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C10" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="D10" s="7" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E10" s="7" t="s">
-        <x:v>208</x:v>
+      <x:c r="D10" s="16" t="str">
+        <x:v>Primary - Weeks 3-4</x:v>
+      </x:c>
+      <x:c r="E10" s="7" t="str">
+        <x:v>Week 3: U2 H1-H5; U2 Apps A-D; Week 4: U2 H6-H13; U2 Apps E-H</x:v>
       </x:c>
       <x:c r="F10" s="7" t="s">
-        <x:v>209</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="G10" s="4"/>
       <x:c r="H10" s="4"/>
       <x:c r="I10" s="4"/>
       <x:c r="J10" s="4"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="7">
         <x:v>6.0</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
-        <x:v>210</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C11" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="D11" s="7" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="E11" s="7" t="s">
-        <x:v>212</x:v>
+      <x:c r="D11" s="16" t="str">
+        <x:v>Primary - Week 5</x:v>
+      </x:c>
+      <x:c r="E11" s="7" t="str">
+        <x:v>Week 5: U3 H1-H3; U3 Apps A-C</x:v>
       </x:c>
       <x:c r="F11" s="7" t="s">
-        <x:v>213</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="G11" s="4"/>
       <x:c r="H11" s="4"/>
       <x:c r="I11" s="4"/>
       <x:c r="J11" s="4"/>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="48" hidden="0" customHeight="1">
       <x:c r="A12" s="7">
         <x:v>7.0</x:v>
       </x:c>
       <x:c r="B12" s="7" t="s">
-        <x:v>214</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C12" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="D12" s="7" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="E12" s="7" t="s">
-        <x:v>215</x:v>
+      <x:c r="D12" s="16" t="str">
+        <x:v>Primary - Week 5; ongoing routine reference in Unit 3 (not a scheduled weekly deck)</x:v>
+      </x:c>
+      <x:c r="E12" s="7" t="str">
+        <x:v>Week 5: U3 H1-H3; U3 Apps A-C</x:v>
       </x:c>
       <x:c r="F12" s="7" t="s">
-        <x:v>216</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="G12" s="4"/>
       <x:c r="H12" s="4"/>
       <x:c r="I12" s="4"/>
       <x:c r="J12" s="4"/>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="36" hidden="0" customHeight="1">
       <x:c r="A13" s="7">
         <x:v>8.0</x:v>
       </x:c>
       <x:c r="B13" s="7" t="s">
-        <x:v>217</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="C13" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="D13" s="7" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="s">
-        <x:v>219</x:v>
+      <x:c r="D13" s="16" t="str">
+        <x:v>Primary - Week 6; Revisit / Reference - Weeks 7, 10, and 13</x:v>
+      </x:c>
+      <x:c r="E13" s="7" t="str">
+        <x:v>Week 6: U3 H4-H5; U3 Apps D-E; Week 7: U3 H6-H7; U3 Apps F-G; Week 10: U3 H11-H12; Week 13: U3 H9, H15</x:v>
       </x:c>
       <x:c r="F13" s="7" t="s">
-        <x:v>220</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="G13" s="4"/>
       <x:c r="H13" s="4"/>
       <x:c r="I13" s="4"/>
       <x:c r="J13" s="4"/>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="36" hidden="0" customHeight="1">
       <x:c r="A14" s="7">
         <x:v>9.0</x:v>
       </x:c>
       <x:c r="B14" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="C14" s="7" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="D14" s="7" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="s">
-        <x:v>224</x:v>
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="str">
+        <x:v>Primary - Weeks 15 and 17; Revisit / Reference - Weeks 9 and 16</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="str">
+        <x:v>Week 9: U3 H9-H10; Week 15: U3 H17; U3 Apps Q-R; Week 16: U3 H18-H19; Week 17: U4 H1-H4; U4 Apps A-C</x:v>
       </x:c>
       <x:c r="F14" s="7" t="s">
-        <x:v>225</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="G14" s="4"/>
       <x:c r="H14" s="4"/>
       <x:c r="I14" s="4"/>
       <x:c r="J14" s="4"/>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="7">
         <x:v>10.0</x:v>
       </x:c>
       <x:c r="B15" s="7" t="s">
-        <x:v>226</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C15" s="7" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="D15" s="7" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="s">
-        <x:v>228</x:v>
+      <x:c r="D15" s="16" t="str">
+        <x:v>Primary - Weeks 17-18</x:v>
+      </x:c>
+      <x:c r="E15" s="7" t="str">
+        <x:v>Week 17: U4 H1-H4; U4 Apps A-C; Week 18: U4 H5-H8; U4 Apps D-G</x:v>
       </x:c>
       <x:c r="F15" s="7" t="s">
-        <x:v>229</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="G15" s="4"/>
       <x:c r="H15" s="4"/>
       <x:c r="I15" s="4"/>
       <x:c r="J15" s="4"/>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="7">
         <x:v>11.0</x:v>
       </x:c>
       <x:c r="B16" s="7" t="s">
-        <x:v>230</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C16" s="7" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="D16" s="7" t="s">
-        <x:v>232</x:v>
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="D16" s="16" t="str">
+        <x:v>Primary - Week 19; Revisit / Reference - Week 24</x:v>
       </x:c>
       <x:c r="E16" s="7" t="str">
-        <x:v>U4 H9-H12; U4 Apps H-K; U5 H5; U5 Apps F-G</x:v>
+        <x:v>Week 19: U4 H9-H12; U4 Apps H-K; Week 24: U5 H5; U5 Apps F-G</x:v>
       </x:c>
       <x:c r="F16" s="7" t="s">
-        <x:v>233</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="G16" s="4"/>
       <x:c r="H16" s="4"/>
       <x:c r="I16" s="4"/>
       <x:c r="J16" s="4"/>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="7">
         <x:v>12.0</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
-        <x:v>234</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="C17" s="7" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="D17" s="7" t="s">
-        <x:v>235</x:v>
+      <x:c r="D17" s="16" t="str">
+        <x:v>Primary - Week 19; Revisit / Reference - Week 20</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
-        <x:v>U4 H11, H13-H17; U4 Apps J, N</x:v>
+        <x:v>Week 19: U4 H9-H12; U4 Apps H-K; Week 20: U4 H13-H17; U4 App N</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
-        <x:v>236</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="G17" s="4"/>
       <x:c r="H17" s="4"/>
       <x:c r="I17" s="4"/>
       <x:c r="J17" s="4"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="36" hidden="0" customHeight="1">
       <x:c r="A18" s="7">
         <x:v>13.0</x:v>
       </x:c>
       <x:c r="B18" s="7" t="s">
-        <x:v>237</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="C18" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="D18" s="7" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="E18" s="7" t="s">
-        <x:v>239</x:v>
+      <x:c r="D18" s="16" t="str">
+        <x:v>Primary - Week 21; Revisit / Reference - Weeks 22, 23, and 26</x:v>
+      </x:c>
+      <x:c r="E18" s="7" t="str">
+        <x:v>Week 21: U5 H1-H2; U5 Apps A, L; Week 22: U5 H3; U5 Apps B-C; Week 23: U5 H4; U5 Apps D-E; Week 26: U5 H7; U5 Apps J-L</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="G18" s="4"/>
       <x:c r="H18" s="4"/>
       <x:c r="I18" s="4"/>
       <x:c r="J18" s="4"/>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="7">
         <x:v>14.0</x:v>
       </x:c>
       <x:c r="B19" s="7" t="s">
-        <x:v>241</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C19" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="D19" s="7" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="E19" s="7" t="s">
-        <x:v>243</x:v>
+      <x:c r="D19" s="16" t="str">
+        <x:v>Primary - Week 25</x:v>
+      </x:c>
+      <x:c r="E19" s="7" t="str">
+        <x:v>Week 25: U5 H6; U5 Apps H-I</x:v>
       </x:c>
       <x:c r="F19" s="7" t="s">
-        <x:v>244</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="G19" s="4"/>
       <x:c r="H19" s="4"/>
       <x:c r="I19" s="4"/>
       <x:c r="J19" s="4"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="7">
         <x:v>15.0</x:v>
       </x:c>
       <x:c r="B20" s="7" t="s">
-        <x:v>245</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="C20" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="D20" s="7" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="E20" s="7" t="s">
-        <x:v>247</x:v>
+      <x:c r="D20" s="16" t="str">
+        <x:v>Primary - Week 27</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="str">
+        <x:v>Week 27: U5 H8-H9; U5 Apps M-N</x:v>
       </x:c>
       <x:c r="F20" s="7" t="s">
-        <x:v>248</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="G20" s="4"/>
       <x:c r="H20" s="4"/>
       <x:c r="I20" s="4"/>
       <x:c r="J20" s="4"/>
     </x:row>
-    <x:row r="21" ht="15.75" customHeight="1">
+    <x:row r="21" ht="24" hidden="0" customHeight="1">
       <x:c r="A21" s="7">
         <x:v>16.0</x:v>
       </x:c>
       <x:c r="B21" s="7" t="s">
-        <x:v>249</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="C21" s="7" t="s">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="D21" s="7" t="s">
-        <x:v>251</x:v>
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="D21" s="16" t="str">
+        <x:v>Primary - Week 28; Revisit / Reference - Week 32</x:v>
       </x:c>
       <x:c r="E21" s="7" t="str">
-        <x:v>U5 H10-H11; U5 App O; U6 H10-H12</x:v>
+        <x:v>Week 28: U5 H10-H11; U5 App O; Week 32: U6 H10-H12</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
-        <x:v>252</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="G21" s="4"/>
       <x:c r="H21" s="4"/>
       <x:c r="I21" s="4"/>
       <x:c r="J21" s="4"/>
     </x:row>
-    <x:row r="22" ht="15.75" customHeight="1">
+    <x:row r="22" ht="48" hidden="0" customHeight="1">
       <x:c r="A22" s="7">
         <x:v>17.0</x:v>
       </x:c>
       <x:c r="B22" s="7" t="s">
-        <x:v>253</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C22" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D22" s="7" t="s">
-        <x:v>254</x:v>
+      <x:c r="D22" s="16" t="str">
+        <x:v>Preview / Reference - Week 28; Primary - Week 29; Revisit / Reference - Week 30</x:v>
       </x:c>
       <x:c r="E22" s="7" t="str">
-        <x:v>U5 H10-H11; U6 H1-H6; U6 Apps A-E</x:v>
+        <x:v>Week 28: U5 H10-H11; U5 App O; Weeks 29-30: U6 H1-H6; U6 Apps A-E</x:v>
       </x:c>
       <x:c r="F22" s="7" t="s">
-        <x:v>255</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="G22" s="4"/>
       <x:c r="H22" s="4"/>
       <x:c r="I22" s="4"/>
       <x:c r="J22" s="4"/>
     </x:row>
-    <x:row r="23" ht="15.75" customHeight="1">
+    <x:row r="23" ht="24" hidden="0" customHeight="1">
       <x:c r="A23" s="7">
         <x:v>18.0</x:v>
       </x:c>
       <x:c r="B23" s="7" t="s">
-        <x:v>256</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C23" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D23" s="7" t="s">
-        <x:v>257</x:v>
-      </x:c>
-      <x:c r="E23" s="7" t="s">
-        <x:v>258</x:v>
+      <x:c r="D23" s="16" t="str">
+        <x:v>Primary - Week 31; Revisit / Reference - Week 32</x:v>
+      </x:c>
+      <x:c r="E23" s="7" t="str">
+        <x:v>Week 31: U6 H7-H9; U6 Apps F-H; Week 32: U6 H10-H12</x:v>
       </x:c>
       <x:c r="F23" s="7" t="s">
-        <x:v>259</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G23" s="4"/>
       <x:c r="H23" s="4"/>
       <x:c r="I23" s="4"/>
       <x:c r="J23" s="4"/>
     </x:row>
-    <x:row r="24" ht="15.75" customHeight="1">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="7">
         <x:v>19.0</x:v>
       </x:c>
       <x:c r="B24" s="7" t="s">
-        <x:v>260</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C24" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D24" s="7" t="s">
-        <x:v>261</x:v>
+      <x:c r="D24" s="16" t="str">
+        <x:v>Primary - Week 34</x:v>
       </x:c>
       <x:c r="E24" s="7" t="str">
-        <x:v>U6 H15-H16, H18</x:v>
+        <x:v>Week 34: U6 H15-H16, H18</x:v>
       </x:c>
       <x:c r="F24" s="7" t="s">
-        <x:v>262</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="G24" s="4"/>
       <x:c r="H24" s="4"/>
@@ -8075,7 +7925,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff0622860f34dfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fbf688b67b543f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8095,12 +7945,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>263</x:v>
+        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>264</x:v>
+        <x:v>205</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -8126,16 +7976,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>265</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>266</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
-        <x:v>267</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="F5" s="6" t="s">
-        <x:v>268</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
@@ -10042,7 +9892,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra43aeb6dc8854a00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redb8c45a072448ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10060,12 +9910,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>269</x:v>
+        <x:v>210</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>270</x:v>
+        <x:v>211</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -10085,16 +9935,16 @@
     </x:row>
     <x:row r="5" ht="31.5" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>271</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>272</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>273</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>274</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
         <x:v>9</x:v>
@@ -10107,16 +9957,16 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="s">
-        <x:v>193</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>275</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
-        <x:v>276</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
-        <x:v>277</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="E6" s="7" t="s">
         <x:v>15</x:v>
@@ -10129,16 +9979,16 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7" t="s">
-        <x:v>197</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
-        <x:v>278</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="C7" s="7" t="s">
-        <x:v>279</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="D7" s="7" t="s">
-        <x:v>280</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="E7" s="7" t="s">
         <x:v>15</x:v>
@@ -10151,10 +10001,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7" t="s">
-        <x:v>281</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
-        <x:v>282</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
         <x:v>Students hold an exact Project Approval Tracker status and have concrete next steps</x:v>
@@ -10173,16 +10023,16 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7" t="s">
-        <x:v>211</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
-        <x:v>283</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>284</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="D9" s="7" t="s">
-        <x:v>285</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="E9" s="7" t="s">
         <x:v>27</x:v>
@@ -10195,16 +10045,16 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7" t="s">
-        <x:v>286</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="B10" s="7" t="s">
-        <x:v>287</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
         <x:v>Students revise, retest, or receive Approved for Systematic Data Collection in the tracker</x:v>
       </x:c>
       <x:c r="D10" s="7" t="s">
-        <x:v>288</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="E10" s="7" t="s">
         <x:v>27</x:v>
@@ -10217,13 +10067,13 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7" t="s">
-        <x:v>289</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
-        <x:v>290</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="C11" s="7" t="s">
-        <x:v>291</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="D11" s="7" t="str">
         <x:v>Record Approved for Systematic Data Collection before full collection begins</x:v>
@@ -10239,16 +10089,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7" t="s">
-        <x:v>292</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="B12" s="7" t="s">
-        <x:v>293</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="C12" s="7" t="s">
-        <x:v>294</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="D12" s="7" t="s">
-        <x:v>295</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="E12" s="7" t="s">
         <x:v>27</x:v>
@@ -10261,16 +10111,16 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="7" t="s">
-        <x:v>296</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="B13" s="7" t="s">
-        <x:v>297</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="C13" s="7" t="s">
-        <x:v>298</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="D13" s="7" t="s">
-        <x:v>299</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="E13" s="7" t="s">
         <x:v>27</x:v>
@@ -10283,16 +10133,16 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7" t="s">
-        <x:v>300</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="B14" s="7" t="s">
-        <x:v>301</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="C14" s="7" t="s">
-        <x:v>302</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="D14" s="7" t="s">
-        <x:v>303</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="E14" s="7" t="s">
         <x:v>33</x:v>
@@ -10305,16 +10155,16 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7" t="s">
-        <x:v>304</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="B15" s="7" t="s">
-        <x:v>305</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="C15" s="7" t="s">
-        <x:v>306</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="D15" s="7" t="s">
-        <x:v>307</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="E15" s="7" t="s">
         <x:v>33</x:v>
@@ -10327,16 +10177,16 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7" t="s">
-        <x:v>308</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="B16" s="7" t="s">
-        <x:v>309</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="C16" s="7" t="s">
-        <x:v>310</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="D16" s="7" t="s">
-        <x:v>311</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="E16" s="7" t="s">
         <x:v>33</x:v>
@@ -10349,16 +10199,16 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7" t="s">
-        <x:v>312</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
-        <x:v>313</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C17" s="7" t="s">
-        <x:v>314</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="D17" s="7" t="s">
-        <x:v>315</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="E17" s="7" t="s">
         <x:v>33</x:v>
@@ -10371,13 +10221,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="7" t="s">
-        <x:v>238</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
         <x:v>Report and public showcase planning launch</x:v>
       </x:c>
       <x:c r="C18" s="7" t="s">
-        <x:v>316</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
         <x:v>Set public format, target date, audience, and space six to eight weeks ahead</x:v>
@@ -10393,16 +10243,16 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="7" t="s">
-        <x:v>317</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="B19" s="7" t="s">
-        <x:v>318</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="C19" s="7" t="s">
-        <x:v>319</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="D19" s="7" t="s">
-        <x:v>320</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="E19" s="7" t="s">
         <x:v>39</x:v>
@@ -10415,16 +10265,16 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="7" t="s">
-        <x:v>246</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="B20" s="7" t="s">
-        <x:v>321</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="C20" s="7" t="s">
-        <x:v>322</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
-        <x:v>323</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="E20" s="7" t="s">
         <x:v>39</x:v>
@@ -10437,13 +10287,13 @@
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="7" t="s">
-        <x:v>324</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="B21" s="7" t="str">
         <x:v>Presentation product and event readiness</x:v>
       </x:c>
       <x:c r="C21" s="7" t="s">
-        <x:v>325</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="D21" s="7" t="str">
         <x:v>Check readability and presentation story; finalize public event logistics</x:v>
@@ -10459,16 +10309,16 @@
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
       <x:c r="A22" s="7" t="s">
-        <x:v>257</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="B22" s="7" t="s">
-        <x:v>326</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="C22" s="7" t="s">
-        <x:v>327</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="D22" s="7" t="s">
-        <x:v>328</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="E22" s="7" t="s">
         <x:v>45</x:v>
@@ -10481,16 +10331,16 @@
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="7" t="s">
-        <x:v>329</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="B23" s="7" t="s">
-        <x:v>330</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="C23" s="7" t="s">
-        <x:v>331</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="D23" s="7" t="s">
-        <x:v>332</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="E23" s="7" t="s">
         <x:v>45</x:v>
@@ -10503,7 +10353,7 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="7" t="s">
-        <x:v>333</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
         <x:v>Required public presentation/showcase</x:v>
@@ -10525,16 +10375,16 @@
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="7" t="s">
-        <x:v>261</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="B25" s="7" t="s">
-        <x:v>334</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C25" s="7" t="s">
-        <x:v>335</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D25" s="7" t="s">
-        <x:v>336</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="E25" s="7" t="s">
         <x:v>45</x:v>
@@ -12133,7 +11983,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9462c46ee0ad498c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6547a95374e14ddf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12153,12 +12003,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>337</x:v>
+        <x:v>285</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>338</x:v>
+        <x:v>286</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -12176,61 +12026,61 @@
       <x:c r="I4" s="4"/>
       <x:c r="J4" s="4"/>
     </x:row>
-    <x:row r="5" ht="31.5" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="s">
         <x:v>53</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="s">
-        <x:v>56</x:v>
+      <x:c r="C5" s="15" t="str">
+        <x:v>Deck Use</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>339</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
-        <x:v>340</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F5" s="6" t="s">
-        <x:v>341</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
       <x:c r="I5" s="4"/>
       <x:c r="J5" s="4"/>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="7">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>61</x:v>
+      <x:c r="C6" s="16" t="str">
+        <x:v>Primary - Deck 1: Authentic Research Course Launch; Deck 3: Research Ethics, Safety, and Integrity</x:v>
       </x:c>
       <x:c r="D6" s="7" t="str">
         <x:v>U1 H1; U1 H2; U1 H3; U1 H4; U1 App A; U1 App B; U1 App C</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str"/>
       <x:c r="F6" s="7" t="s">
-        <x:v>62</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="G6" s="4"/>
       <x:c r="H6" s="4"/>
       <x:c r="I6" s="4"/>
       <x:c r="J6" s="4"/>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="7">
         <x:v>2.0</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>65</x:v>
+      <x:c r="C7" s="16" t="str">
+        <x:v>Primary - Deck 2: From Topic to Research Question; Deck 4: Experimental &amp; Engineering Design</x:v>
       </x:c>
       <x:c r="D7" s="7" t="str">
         <x:v>U1 H5; U1 H6; U1 H7; U1 H8; U1 App D; U1 App E; U1 App F; U1 App G; U1 App H</x:v>
@@ -12239,44 +12089,44 @@
         <x:v>U1 App I</x:v>
       </x:c>
       <x:c r="F7" s="7" t="s">
-        <x:v>66</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="G7" s="4"/>
       <x:c r="H7" s="4"/>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="36" hidden="0" customHeight="1">
       <x:c r="A8" s="7">
         <x:v>3.0</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="s">
-        <x:v>69</x:v>
+      <x:c r="C8" s="16" t="str">
+        <x:v>Primary - Deck 5: Building a Formal Research Plan; Revisit / Reference - Deck 4: Experimental &amp; Engineering Design</x:v>
       </x:c>
       <x:c r="D8" s="7" t="str">
         <x:v>U2 H1; U2 H2; U2 H3; U2 H4; U2 H5; U2 App A; U2 App B; U2 App C; U2 App D</x:v>
       </x:c>
       <x:c r="E8" s="7" t="str"/>
       <x:c r="F8" s="7" t="s">
-        <x:v>70</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="G8" s="4"/>
       <x:c r="H8" s="4"/>
       <x:c r="I8" s="4"/>
       <x:c r="J8" s="4"/>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="36" hidden="0" customHeight="1">
       <x:c r="A9" s="7">
         <x:v>4.0</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C9" s="7" t="s">
-        <x:v>69</x:v>
+      <x:c r="C9" s="16" t="str">
+        <x:v>Primary - Deck 5: Building a Formal Research Plan; Revisit / Reference - Deck 3: Research Ethics, Safety, and Integrity</x:v>
       </x:c>
       <x:c r="D9" s="7" t="str">
         <x:v>U2 H6; U2 H7; U2 H8; U2 H9; U2 H10; U2 H11; U2 H12; U2 H13; U2 App E; U2 App F; U2 App G; U2 App H</x:v>
@@ -12285,88 +12135,88 @@
         <x:v>U2 AppI; U2 AppJ; district-supplied approval and safety forms as applicable</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
-        <x:v>73</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="G9" s="4"/>
       <x:c r="H9" s="4"/>
       <x:c r="I9" s="4"/>
       <x:c r="J9" s="4"/>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="24" hidden="0" customHeight="1">
       <x:c r="A10" s="7">
         <x:v>5.0</x:v>
       </x:c>
       <x:c r="B10" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>76</x:v>
+      <x:c r="C10" s="16" t="str">
+        <x:v>Primary - Deck 6: Pilot Testing; Deck 7: Research Journals and Documentation</x:v>
       </x:c>
       <x:c r="D10" s="7" t="str">
         <x:v>U3 H1; U3 H2; U3 H3; U3 App A; U3 App B; U3 App C</x:v>
       </x:c>
       <x:c r="E10" s="7" t="str"/>
       <x:c r="F10" s="7" t="s">
-        <x:v>77</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="G10" s="4"/>
       <x:c r="H10" s="4"/>
       <x:c r="I10" s="4"/>
       <x:c r="J10" s="4"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="7">
         <x:v>6.0</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>80</x:v>
+      <x:c r="C11" s="16" t="str">
+        <x:v>Primary - Deck 8: Troubleshooting and Responsible Project Pivots</x:v>
       </x:c>
       <x:c r="D11" s="7" t="str">
         <x:v>U3 H4; U3 H5; U3 App D; U3 App E</x:v>
       </x:c>
       <x:c r="E11" s="7" t="str"/>
       <x:c r="F11" s="7" t="s">
-        <x:v>81</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="G11" s="4"/>
       <x:c r="H11" s="4"/>
       <x:c r="I11" s="4"/>
       <x:c r="J11" s="4"/>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="7">
         <x:v>7.0</x:v>
       </x:c>
       <x:c r="B12" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>84</x:v>
+      <x:c r="C12" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 8</x:v>
       </x:c>
       <x:c r="D12" s="7" t="str">
         <x:v>U3 H6; U3 H7; U3 App F; U3 App G</x:v>
       </x:c>
       <x:c r="E12" s="7" t="str"/>
       <x:c r="F12" s="7" t="s">
-        <x:v>85</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="G12" s="4"/>
       <x:c r="H12" s="4"/>
       <x:c r="I12" s="4"/>
       <x:c r="J12" s="4"/>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="7">
         <x:v>8.0</x:v>
       </x:c>
       <x:c r="B13" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>88</x:v>
+      <x:c r="C13" s="16" t="str">
+        <x:v>No New Deck - systematic data collection work sessions</x:v>
       </x:c>
       <x:c r="D13" s="7" t="str">
         <x:v>U3 H8; U3 H9; U3 App H</x:v>
@@ -12375,22 +12225,22 @@
         <x:v>U3 App I</x:v>
       </x:c>
       <x:c r="F13" s="7" t="s">
-        <x:v>89</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="G13" s="4"/>
       <x:c r="H13" s="4"/>
       <x:c r="I13" s="4"/>
       <x:c r="J13" s="4"/>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="7">
         <x:v>9.0</x:v>
       </x:c>
       <x:c r="B14" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C14" s="7" t="s">
-        <x:v>92</x:v>
+      <x:c r="C14" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 9 as needed</x:v>
       </x:c>
       <x:c r="D14" s="7" t="str">
         <x:v>U3 H9; U3 H10</x:v>
@@ -12399,22 +12249,22 @@
         <x:v>U3 App J</x:v>
       </x:c>
       <x:c r="F14" s="7" t="s">
-        <x:v>93</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="G14" s="4"/>
       <x:c r="H14" s="4"/>
       <x:c r="I14" s="4"/>
       <x:c r="J14" s="4"/>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="7">
         <x:v>10.0</x:v>
       </x:c>
       <x:c r="B15" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>96</x:v>
+      <x:c r="C15" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 8</x:v>
       </x:c>
       <x:c r="D15" s="7" t="str">
         <x:v>U3 H11; U3 H12</x:v>
@@ -12423,22 +12273,22 @@
         <x:v>U3 App K; U3 App L</x:v>
       </x:c>
       <x:c r="F15" s="7" t="s">
-        <x:v>97</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="G15" s="4"/>
       <x:c r="H15" s="4"/>
       <x:c r="I15" s="4"/>
       <x:c r="J15" s="4"/>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="7">
         <x:v>11.0</x:v>
       </x:c>
       <x:c r="B16" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="C16" s="16" t="str">
+        <x:v>No New Deck - data collection and reliability work sessions</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
         <x:v>U3 H9; U3 H13</x:v>
@@ -12447,22 +12297,22 @@
         <x:v>U3 App M</x:v>
       </x:c>
       <x:c r="F16" s="7" t="s">
-        <x:v>101</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="G16" s="4"/>
       <x:c r="H16" s="4"/>
       <x:c r="I16" s="4"/>
       <x:c r="J16" s="4"/>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="7">
         <x:v>12.0</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="C17" s="16" t="str">
+        <x:v>No New Deck - midpoint review and progress reporting</x:v>
       </x:c>
       <x:c r="D17" s="7" t="str">
         <x:v>U3 H14; U3 App N</x:v>
@@ -12471,22 +12321,22 @@
         <x:v>U3 App O</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
-        <x:v>104</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="G17" s="4"/>
       <x:c r="H17" s="4"/>
       <x:c r="I17" s="4"/>
       <x:c r="J17" s="4"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="7">
         <x:v>13.0</x:v>
       </x:c>
       <x:c r="B18" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="C18" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 8 as needed</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
         <x:v>U3 H9; U3 H15</x:v>
@@ -12495,66 +12345,66 @@
         <x:v>U3 App P</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
-        <x:v>107</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="G18" s="4"/>
       <x:c r="H18" s="4"/>
       <x:c r="I18" s="4"/>
       <x:c r="J18" s="4"/>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="24" hidden="0" customHeight="1">
       <x:c r="A19" s="7">
         <x:v>14.0</x:v>
       </x:c>
       <x:c r="B19" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="C19" s="16" t="str">
+        <x:v>No New Deck - major trial or prototype completion work sessions</x:v>
       </x:c>
       <x:c r="D19" s="7" t="str">
         <x:v>U3 H9; U3 H16</x:v>
       </x:c>
       <x:c r="E19" s="7" t="str"/>
       <x:c r="F19" s="7" t="s">
-        <x:v>110</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G19" s="4"/>
       <x:c r="H19" s="4"/>
       <x:c r="I19" s="4"/>
       <x:c r="J19" s="4"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="7">
         <x:v>15.0</x:v>
       </x:c>
       <x:c r="B20" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>113</x:v>
+      <x:c r="C20" s="16" t="str">
+        <x:v>Primary - Deck 9: Data Organization, Raw vs. Clean Data</x:v>
       </x:c>
       <x:c r="D20" s="7" t="str">
         <x:v>U3 H17; U3 App Q; U3 App R</x:v>
       </x:c>
       <x:c r="E20" s="7" t="str"/>
       <x:c r="F20" s="7" t="s">
-        <x:v>114</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="G20" s="4"/>
       <x:c r="H20" s="4"/>
       <x:c r="I20" s="4"/>
       <x:c r="J20" s="4"/>
     </x:row>
-    <x:row r="21" ht="15.75" customHeight="1">
+    <x:row r="21" ht="24" hidden="0" customHeight="1">
       <x:c r="A21" s="7">
         <x:v>16.0</x:v>
       </x:c>
       <x:c r="B21" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C21" s="7" t="s">
-        <x:v>117</x:v>
+      <x:c r="C21" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 9</x:v>
       </x:c>
       <x:c r="D21" s="7" t="str">
         <x:v>U3 H18; U3 H19</x:v>
@@ -12563,88 +12413,88 @@
         <x:v>U3 App S; U3 App T; U3 App U</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
-        <x:v>118</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="G21" s="4"/>
       <x:c r="H21" s="4"/>
       <x:c r="I21" s="4"/>
       <x:c r="J21" s="4"/>
     </x:row>
-    <x:row r="22" ht="15.75" customHeight="1">
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
       <x:c r="A22" s="7">
         <x:v>17.0</x:v>
       </x:c>
       <x:c r="B22" s="7" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>121</x:v>
+      <x:c r="C22" s="16" t="str">
+        <x:v>Primary - Deck 9: Data Organization; Deck 10: Choosing the Right Analysis Method</x:v>
       </x:c>
       <x:c r="D22" s="7" t="str">
         <x:v>U4 H1; U4 H2; U4 H3; U4 H4; U4 App A; U4 App B; U4 App C</x:v>
       </x:c>
       <x:c r="E22" s="7" t="str"/>
       <x:c r="F22" s="7" t="s">
-        <x:v>122</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="G22" s="4"/>
       <x:c r="H22" s="4"/>
       <x:c r="I22" s="4"/>
       <x:c r="J22" s="4"/>
     </x:row>
-    <x:row r="23" ht="15.75" customHeight="1">
+    <x:row r="23" ht="24" hidden="0" customHeight="1">
       <x:c r="A23" s="7">
         <x:v>18.0</x:v>
       </x:c>
       <x:c r="B23" s="7" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>125</x:v>
+      <x:c r="C23" s="16" t="str">
+        <x:v>Primary - Deck 10: Choosing the Right Analysis Method</x:v>
       </x:c>
       <x:c r="D23" s="7" t="str">
         <x:v>U4 H5; U4 H6; U4 H7; U4 H8; U4 App D; U4 App E; U4 App F; U4 App G</x:v>
       </x:c>
       <x:c r="E23" s="7" t="str"/>
       <x:c r="F23" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="G23" s="4"/>
       <x:c r="H23" s="4"/>
       <x:c r="I23" s="4"/>
       <x:c r="J23" s="4"/>
     </x:row>
-    <x:row r="24" ht="15.75" customHeight="1">
+    <x:row r="24" ht="24" hidden="0" customHeight="1">
       <x:c r="A24" s="7">
         <x:v>19.0</x:v>
       </x:c>
       <x:c r="B24" s="7" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="C24" s="7" t="s">
-        <x:v>129</x:v>
+      <x:c r="C24" s="16" t="str">
+        <x:v>Primary - Deck 11: Graphing and Visual Ethics; Deck 12: Error, Uncertainty, and Limitations</x:v>
       </x:c>
       <x:c r="D24" s="7" t="str">
         <x:v>U4 H9; U4 H10; U4 H11; U4 H12; U4 App H; U4 App I; U4 App J; U4 App K</x:v>
       </x:c>
       <x:c r="E24" s="7" t="str"/>
       <x:c r="F24" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="G24" s="4"/>
       <x:c r="H24" s="4"/>
       <x:c r="I24" s="4"/>
       <x:c r="J24" s="4"/>
     </x:row>
-    <x:row r="25" ht="15.75" customHeight="1">
+    <x:row r="25" ht="24" hidden="0" customHeight="1">
       <x:c r="A25" s="7">
         <x:v>20.0</x:v>
       </x:c>
       <x:c r="B25" s="7" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="C25" s="7" t="s">
-        <x:v>133</x:v>
+      <x:c r="C25" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 12</x:v>
       </x:c>
       <x:c r="D25" s="7" t="str">
         <x:v>U4 H13; U4 H14; U4 H15; U4 H16; U4 H17; U4 App N</x:v>
@@ -12653,176 +12503,176 @@
         <x:v>U4 App L; U4 App M; U4 App O; U4 App P; U4 App Q</x:v>
       </x:c>
       <x:c r="F25" s="7" t="s">
-        <x:v>134</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="G25" s="4"/>
       <x:c r="H25" s="4"/>
       <x:c r="I25" s="4"/>
       <x:c r="J25" s="4"/>
     </x:row>
-    <x:row r="26" ht="15.75" customHeight="1">
+    <x:row r="26" ht="24" hidden="0" customHeight="1">
       <x:c r="A26" s="7">
         <x:v>21.0</x:v>
       </x:c>
       <x:c r="B26" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C26" s="7" t="s">
-        <x:v>137</x:v>
+      <x:c r="C26" s="16" t="str">
+        <x:v>Primary - Deck 13: Scientific Report Structure</x:v>
       </x:c>
       <x:c r="D26" s="7" t="str">
         <x:v>U5 H1; U5 H2; U5 App A; U5 App L</x:v>
       </x:c>
       <x:c r="E26" s="7" t="str"/>
       <x:c r="F26" s="7" t="s">
-        <x:v>138</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="G26" s="4"/>
       <x:c r="H26" s="4"/>
       <x:c r="I26" s="4"/>
       <x:c r="J26" s="4"/>
     </x:row>
-    <x:row r="27" ht="15.75" customHeight="1">
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="7">
         <x:v>22.0</x:v>
       </x:c>
       <x:c r="B27" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>140</x:v>
+      <x:c r="C27" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 13</x:v>
       </x:c>
       <x:c r="D27" s="7" t="str">
         <x:v>U5 H3; U5 App B; U5 App C</x:v>
       </x:c>
       <x:c r="E27" s="7" t="str"/>
       <x:c r="F27" s="7" t="s">
-        <x:v>141</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G27" s="4"/>
       <x:c r="H27" s="4"/>
       <x:c r="I27" s="4"/>
       <x:c r="J27" s="4"/>
     </x:row>
-    <x:row r="28" ht="15.75" customHeight="1">
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="7">
         <x:v>23.0</x:v>
       </x:c>
       <x:c r="B28" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>140</x:v>
+      <x:c r="C28" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 13</x:v>
       </x:c>
       <x:c r="D28" s="7" t="str">
         <x:v>U5 H4; U5 App D; U5 App E</x:v>
       </x:c>
       <x:c r="E28" s="7" t="str"/>
       <x:c r="F28" s="7" t="s">
-        <x:v>144</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="G28" s="4"/>
       <x:c r="H28" s="4"/>
       <x:c r="I28" s="4"/>
       <x:c r="J28" s="4"/>
     </x:row>
-    <x:row r="29" ht="15.75" customHeight="1">
+    <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="7">
         <x:v>24.0</x:v>
       </x:c>
       <x:c r="B29" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>147</x:v>
+      <x:c r="C29" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 11</x:v>
       </x:c>
       <x:c r="D29" s="7" t="str">
         <x:v>U5 H5; U5 App F; U5 App G</x:v>
       </x:c>
       <x:c r="E29" s="7" t="str"/>
       <x:c r="F29" s="7" t="s">
-        <x:v>148</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="G29" s="4"/>
       <x:c r="H29" s="4"/>
       <x:c r="I29" s="4"/>
       <x:c r="J29" s="4"/>
     </x:row>
-    <x:row r="30" ht="15.75" customHeight="1">
+    <x:row r="30" ht="24" hidden="0" customHeight="1">
       <x:c r="A30" s="7">
         <x:v>25.0</x:v>
       </x:c>
       <x:c r="B30" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C30" s="7" t="s">
-        <x:v>150</x:v>
+      <x:c r="C30" s="16" t="str">
+        <x:v>Primary - Deck 14: Writing the Discussion with CER</x:v>
       </x:c>
       <x:c r="D30" s="7" t="str">
         <x:v>U5 H6; U5 App H; U5 App I</x:v>
       </x:c>
       <x:c r="E30" s="7" t="str"/>
       <x:c r="F30" s="7" t="s">
-        <x:v>151</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="G30" s="4"/>
       <x:c r="H30" s="4"/>
       <x:c r="I30" s="4"/>
       <x:c r="J30" s="4"/>
     </x:row>
-    <x:row r="31" ht="15.75" customHeight="1">
+    <x:row r="31" ht="24" hidden="0" customHeight="1">
       <x:c r="A31" s="7">
         <x:v>26.0</x:v>
       </x:c>
       <x:c r="B31" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C31" s="7" t="s">
-        <x:v>154</x:v>
+      <x:c r="C31" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 13</x:v>
       </x:c>
       <x:c r="D31" s="7" t="str">
         <x:v>U5 H7; U5 App J; U5 App K; U5 App L</x:v>
       </x:c>
       <x:c r="E31" s="7" t="str"/>
       <x:c r="F31" s="7" t="s">
-        <x:v>155</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="G31" s="4"/>
       <x:c r="H31" s="4"/>
       <x:c r="I31" s="4"/>
       <x:c r="J31" s="4"/>
     </x:row>
-    <x:row r="32" ht="15.75" customHeight="1">
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="7">
         <x:v>27.0</x:v>
       </x:c>
       <x:c r="B32" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C32" s="7" t="s">
-        <x:v>158</x:v>
+      <x:c r="C32" s="16" t="str">
+        <x:v>Primary - Deck 15: Peer Review and Scientific Revision</x:v>
       </x:c>
       <x:c r="D32" s="7" t="str">
         <x:v>U5 H8; U5 H9; U5 App M; U5 App N</x:v>
       </x:c>
       <x:c r="E32" s="7" t="str"/>
       <x:c r="F32" s="7" t="s">
-        <x:v>159</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="G32" s="4"/>
       <x:c r="H32" s="4"/>
       <x:c r="I32" s="4"/>
       <x:c r="J32" s="4"/>
     </x:row>
-    <x:row r="33" ht="15.75" customHeight="1">
+    <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="7">
         <x:v>28.0</x:v>
       </x:c>
       <x:c r="B33" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C33" s="7" t="s">
-        <x:v>161</x:v>
+      <x:c r="C33" s="16" t="str">
+        <x:v>Primary - Deck 16: Designing a Research Poster/Board; Preview / Reference - Deck 17</x:v>
       </x:c>
       <x:c r="D33" s="7" t="str">
         <x:v>U5 H10; U5 H11; U5 App O</x:v>
@@ -12831,88 +12681,88 @@
         <x:v>U5 App Q</x:v>
       </x:c>
       <x:c r="F33" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="G33" s="4"/>
       <x:c r="H33" s="4"/>
       <x:c r="I33" s="4"/>
       <x:c r="J33" s="4"/>
     </x:row>
-    <x:row r="34" ht="15.75" customHeight="1">
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
       <x:c r="A34" s="7">
         <x:v>29.0</x:v>
       </x:c>
       <x:c r="B34" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>165</x:v>
+      <x:c r="C34" s="16" t="str">
+        <x:v>Primary - Deck 17: Oral Presentation Skills for Research</x:v>
       </x:c>
       <x:c r="D34" s="7" t="str">
         <x:v>U6 H1; U6 H2; U6 H3; U6 App A; U6 App B; U6 App C</x:v>
       </x:c>
       <x:c r="E34" s="7" t="str"/>
       <x:c r="F34" s="7" t="s">
-        <x:v>166</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="G34" s="4"/>
       <x:c r="H34" s="4"/>
       <x:c r="I34" s="4"/>
       <x:c r="J34" s="4"/>
     </x:row>
-    <x:row r="35" ht="15.75" customHeight="1">
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
       <x:c r="A35" s="7">
         <x:v>30.0</x:v>
       </x:c>
       <x:c r="B35" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C35" s="7" t="s">
-        <x:v>169</x:v>
+      <x:c r="C35" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Deck 17</x:v>
       </x:c>
       <x:c r="D35" s="7" t="str">
         <x:v>U6 H4; U6 H5; U6 H6; U6 App D; U6 App E</x:v>
       </x:c>
       <x:c r="E35" s="7" t="str"/>
       <x:c r="F35" s="7" t="s">
-        <x:v>170</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="G35" s="4"/>
       <x:c r="H35" s="4"/>
       <x:c r="I35" s="4"/>
       <x:c r="J35" s="4"/>
     </x:row>
-    <x:row r="36" ht="15.75" customHeight="1">
+    <x:row r="36" ht="24" hidden="0" customHeight="1">
       <x:c r="A36" s="7">
         <x:v>31.0</x:v>
       </x:c>
       <x:c r="B36" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C36" s="7" t="s">
-        <x:v>173</x:v>
+      <x:c r="C36" s="16" t="str">
+        <x:v>Primary - Deck 18: Answering Questions Like a Scientist</x:v>
       </x:c>
       <x:c r="D36" s="7" t="str">
         <x:v>U6 H7; U6 H8; U6 H9; U6 App F; U6 App G; U6 App H</x:v>
       </x:c>
       <x:c r="E36" s="7" t="str"/>
       <x:c r="F36" s="7" t="s">
-        <x:v>174</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="G36" s="4"/>
       <x:c r="H36" s="4"/>
       <x:c r="I36" s="4"/>
       <x:c r="J36" s="4"/>
     </x:row>
-    <x:row r="37" ht="15.75" customHeight="1">
+    <x:row r="37" ht="24" hidden="0" customHeight="1">
       <x:c r="A37" s="7">
         <x:v>32.0</x:v>
       </x:c>
       <x:c r="B37" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>177</x:v>
+      <x:c r="C37" s="16" t="str">
+        <x:v>No New Deck; Revisit / Reference - Decks 16 and 18</x:v>
       </x:c>
       <x:c r="D37" s="7" t="str">
         <x:v>U6 H10; U6 H11; U6 H12</x:v>
@@ -12921,22 +12771,22 @@
         <x:v>U6 App I; U6 App J; U6 App K</x:v>
       </x:c>
       <x:c r="F37" s="7" t="s">
-        <x:v>178</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="G37" s="4"/>
       <x:c r="H37" s="4"/>
       <x:c r="I37" s="4"/>
       <x:c r="J37" s="4"/>
     </x:row>
-    <x:row r="38" ht="15.75" customHeight="1">
+    <x:row r="38" ht="24" hidden="0" customHeight="1">
       <x:c r="A38" s="7">
         <x:v>33.0</x:v>
       </x:c>
       <x:c r="B38" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C38" s="7" t="s">
-        <x:v>100</x:v>
+      <x:c r="C38" s="16" t="str">
+        <x:v>No New Deck - required public presentation or showcase</x:v>
       </x:c>
       <x:c r="D38" s="7" t="str">
         <x:v>U6 H13; U6 H14; U6 App L; U6 App M</x:v>
@@ -12945,22 +12795,22 @@
         <x:v>U6 App N</x:v>
       </x:c>
       <x:c r="F38" s="7" t="s">
-        <x:v>342</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="G38" s="4"/>
       <x:c r="H38" s="4"/>
       <x:c r="I38" s="4"/>
       <x:c r="J38" s="4"/>
     </x:row>
-    <x:row r="39" ht="15.75" customHeight="1">
+    <x:row r="39" ht="24" hidden="0" customHeight="1">
       <x:c r="A39" s="7">
         <x:v>34.0</x:v>
       </x:c>
       <x:c r="B39" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>181</x:v>
+      <x:c r="C39" s="16" t="str">
+        <x:v>Primary - Deck 19: Final Reflection and Research Portfolio</x:v>
       </x:c>
       <x:c r="D39" s="7" t="str">
         <x:v>U6 H15; U6 H16; U6 H18</x:v>
@@ -12969,7 +12819,7 @@
         <x:v>U6 H17; U6 App O; U6 App P; U6 App Q; U6 App R; U6 App S</x:v>
       </x:c>
       <x:c r="F39" s="7" t="s">
-        <x:v>182</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="G39" s="4"/>
       <x:c r="H39" s="4"/>
@@ -14396,7 +14246,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0796fde07f474bde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67f6c047978e4cbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Align weekly support resource mappings
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
+++ b/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R3030208b8d9644ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="R30b31aa5c77b4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="R337fca7f276047c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R998a303668614c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="R320c77bcd1c24532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="Rd0a7cd389bb44bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R65be224c0ae1428e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="Rb616e6b4b1944c56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="Rdb3db2c035514e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R10f67599e3954b84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="R2bb4c2568c174fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="R8eb035c0a96f4dd9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -486,147 +486,6 @@
     <x:t xml:space="preserve">STARLAB Slide Deck Alignment</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Deck sequence, unit/week connection, and required print materials</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Deck #</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Deck Title</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Primary Unit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Instructional Purpose</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Authentic Research Course Launch</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Course launch and STARLAB identity</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">From Topic to Research Question</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Topic narrowing and question quality</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Research Ethics, Safety, and Integrity</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 1 / Unit 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ethics, safety, and approval culture</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Experimental &amp; Engineering Design Basics</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Variables, controls, criteria, constraints</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Building a Formal Research Plan</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Formal research planning and approval</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Pilot Testing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Testing small before full data collection</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Research Journals and Documentation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Journal setup and scientific documentation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Troubleshooting and Responsible Project Pivots</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Diagnose, revise, document, pivot responsibly</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Data Organization: Raw Data vs. Clean Data</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 / Unit 4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Preserve raw data and create clean copies</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Choosing the Right Data Analysis Method</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Match data type to analysis method</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Graphing and Visual Ethics</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 4 / Unit 5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Clear, honest data visuals</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Error, Uncertainty, and Limitations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Interpret evidence with caution</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Scientific Report Structure</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Report architecture and planning</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Writing the Discussion: CER</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Claim-evidence-reasoning, limitations, future work</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Peer Review and Scientific Revision</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Structured feedback and revision</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Designing a Research Poster or Presentation Board</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 5 / Unit 6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visual aid and showcase preparation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Oral Presentation Skills for Research</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Research story, speaking notes, practice</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Answering Questions Like a Scientist</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Q&amp;A, evidence defense, scientific humility</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Final Reflection and Research Portfolio</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Portfolio, reflection, continuation planning</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Unit Overview and Portal Placement</x:t>
   </x:si>
   <x:si>
@@ -892,7 +751,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF000000"/>
@@ -932,8 +791,41 @@
       <x:color theme="1"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -970,14 +862,123 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF050505"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFED1C24"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="8">
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC8141B"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFC8141B"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFC8141B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC8141B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7EEF7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF73C8E6"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -1027,6 +1028,150 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3321,7 +3466,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26f1583fba4047bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74314cd53b5741f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3424,7 +3569,9 @@
       <x:c r="I6" s="7" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="J6" s="13" t="str"/>
+      <x:c r="J6" s="13" t="str">
+        <x:v>U1 App I; U1 App J; U1 App L</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="7">
@@ -3453,7 +3600,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="J7" s="14" t="str">
-        <x:v>U1 App I</x:v>
+        <x:v>U1 App I; U1 App K</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" hidden="0" customHeight="1">
@@ -3482,7 +3629,9 @@
       <x:c r="I8" s="7" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="J8" s="13" t="str"/>
+      <x:c r="J8" s="13" t="str">
+        <x:v>U2 App K</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="36" hidden="0" customHeight="1">
       <x:c r="A9" s="7">
@@ -3511,7 +3660,7 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str">
-        <x:v>U2 AppI; U2 AppJ; district-supplied approval and safety forms as applicable</x:v>
+        <x:v>U2 App I; U2 App J; U2 App L; district-supplied approval and safety forms as applicable</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" hidden="0" customHeight="1">
@@ -3540,7 +3689,7 @@
       <x:c r="I10" s="7" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="J10" s="13" t="str"/>
+      <x:c r="J10" s="13"/>
     </x:row>
     <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="7">
@@ -3568,7 +3717,7 @@
       <x:c r="I11" s="7" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="J11" s="14" t="str"/>
+      <x:c r="J11" s="14"/>
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="7">
@@ -3596,7 +3745,7 @@
       <x:c r="I12" s="7" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="J12" s="13" t="str"/>
+      <x:c r="J12" s="13"/>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="7">
@@ -3804,7 +3953,7 @@
       <x:c r="I19" s="7" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="J19" s="14" t="str"/>
+      <x:c r="J19" s="14"/>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="7">
@@ -3832,7 +3981,7 @@
       <x:c r="I20" s="7" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="J20" s="13" t="str"/>
+      <x:c r="J20" s="13"/>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
       <x:c r="A21" s="7">
@@ -3890,7 +4039,7 @@
       <x:c r="I22" s="7" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="J22" s="13" t="str"/>
+      <x:c r="J22" s="13"/>
     </x:row>
     <x:row r="23" ht="24" hidden="0" customHeight="1">
       <x:c r="A23" s="7">
@@ -3918,7 +4067,7 @@
       <x:c r="I23" s="7" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="J23" s="14" t="str"/>
+      <x:c r="J23" s="14"/>
     </x:row>
     <x:row r="24" ht="24" hidden="0" customHeight="1">
       <x:c r="A24" s="7">
@@ -3946,7 +4095,7 @@
       <x:c r="I24" s="7" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="J24" s="13" t="str"/>
+      <x:c r="J24" s="13"/>
     </x:row>
     <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="7">
@@ -4004,7 +4153,9 @@
       <x:c r="I26" s="7" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="J26" s="13" t="str"/>
+      <x:c r="J26" s="13" t="str">
+        <x:v>U5 App R; U5 App S</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="24" hidden="0" customHeight="1">
       <x:c r="A27" s="7">
@@ -4032,7 +4183,7 @@
       <x:c r="I27" s="7" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="J27" s="14" t="str"/>
+      <x:c r="J27" s="14"/>
     </x:row>
     <x:row r="28" ht="24" hidden="0" customHeight="1">
       <x:c r="A28" s="7">
@@ -4060,7 +4211,7 @@
       <x:c r="I28" s="7" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="J28" s="13" t="str"/>
+      <x:c r="J28" s="13"/>
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="7">
@@ -4088,7 +4239,7 @@
       <x:c r="I29" s="7" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="J29" s="14" t="str"/>
+      <x:c r="J29" s="14"/>
     </x:row>
     <x:row r="30" ht="24" hidden="0" customHeight="1">
       <x:c r="A30" s="7">
@@ -4116,7 +4267,7 @@
       <x:c r="I30" s="7" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="J30" s="13" t="str"/>
+      <x:c r="J30" s="13"/>
     </x:row>
     <x:row r="31" ht="24" hidden="0" customHeight="1">
       <x:c r="A31" s="7">
@@ -4144,7 +4295,7 @@
       <x:c r="I31" s="7" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="J31" s="14" t="str"/>
+      <x:c r="J31" s="14"/>
     </x:row>
     <x:row r="32" ht="24" hidden="0" customHeight="1">
       <x:c r="A32" s="7">
@@ -4172,7 +4323,7 @@
       <x:c r="I32" s="7" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="J32" s="13" t="str"/>
+      <x:c r="J32" s="13"/>
     </x:row>
     <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="7">
@@ -4201,7 +4352,7 @@
         <x:v>140</x:v>
       </x:c>
       <x:c r="J33" s="14" t="str">
-        <x:v>U5 App Q</x:v>
+        <x:v>U5 App Q; U6 App L</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="24" hidden="0" customHeight="1">
@@ -4230,7 +4381,9 @@
       <x:c r="I34" s="7" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="J34" s="13" t="str"/>
+      <x:c r="J34" s="13" t="str">
+        <x:v>U6 App L</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="24" hidden="0" customHeight="1">
       <x:c r="A35" s="7">
@@ -4258,7 +4411,9 @@
       <x:c r="I35" s="7" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="J35" s="14" t="str"/>
+      <x:c r="J35" s="14" t="str">
+        <x:v>U6 App L</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="24" hidden="0" customHeight="1">
       <x:c r="A36" s="7">
@@ -4286,7 +4441,9 @@
       <x:c r="I36" s="7" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="J36" s="13" t="str"/>
+      <x:c r="J36" s="13" t="str">
+        <x:v>U6 App L</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="24" hidden="0" customHeight="1">
       <x:c r="A37" s="7">
@@ -4315,7 +4472,7 @@
         <x:v>152</x:v>
       </x:c>
       <x:c r="J37" s="14" t="str">
-        <x:v>U6 App I; U6 App J; U6 App K</x:v>
+        <x:v>U6 App I; U6 App J; U6 App K; U6 App L</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="36" hidden="0" customHeight="1">
@@ -5803,7 +5960,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34cebcbc746c4c61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cedb62434d44ae9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5812,28 +5969,53 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultColWidth="12.630000114440918" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" customWidth="1"/>
-    <x:col min="2" max="2" width="42" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="4" width="18" customWidth="1"/>
-    <x:col min="5" max="5" width="55" customWidth="1"/>
-    <x:col min="6" max="6" width="45" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="46" hidden="0" customWidth="1"/>
     <x:col min="7" max="26" width="8.630000114440918" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="39" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="1" t="s">
+    <x:row r="1" ht="28" hidden="0" customHeight="1">
+      <x:c r="A1" s="17" t="s">
         <x:v>156</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="2" t="s">
-        <x:v>157</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="3"/>
-    </x:row>
-    <x:row r="4">
+      <x:c r="B1" s="22"/>
+      <x:c r="C1" s="22"/>
+      <x:c r="D1" s="22"/>
+      <x:c r="E1" s="22"/>
+      <x:c r="F1" s="22"/>
+      <x:c r="G1" s="22"/>
+      <x:c r="H1" s="22"/>
+    </x:row>
+    <x:row r="2" ht="34" hidden="0" customHeight="1">
+      <x:c r="A2" s="19" t="str">
+        <x:v>Rows are ordered by deck number, not chronologically. Read Primary Use first; later use appears in the Preview / Revisit / Reference column.</x:v>
+      </x:c>
+      <x:c r="B2" s="22"/>
+      <x:c r="C2" s="22"/>
+      <x:c r="D2" s="22"/>
+      <x:c r="E2" s="22"/>
+      <x:c r="F2" s="22"/>
+      <x:c r="G2" s="22"/>
+      <x:c r="H2" s="22"/>
+    </x:row>
+    <x:row r="3" ht="10" hidden="0" customHeight="1">
+      <x:c r="A3" s="23"/>
+      <x:c r="B3" s="24"/>
+      <x:c r="C3" s="24"/>
+      <x:c r="D3" s="24"/>
+      <x:c r="E3" s="24"/>
+      <x:c r="F3" s="24"/>
+      <x:c r="G3" s="24"/>
+      <x:c r="H3" s="24"/>
+    </x:row>
+    <x:row r="4" ht="8" hidden="0" customHeight="1">
       <x:c r="A4" s="4"/>
       <x:c r="B4" s="4"/>
       <x:c r="C4" s="4"/>
@@ -5845,483 +6027,564 @@
       <x:c r="I4" s="4"/>
       <x:c r="J4" s="4"/>
     </x:row>
-    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A5" s="6" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="D5" s="15" t="str">
-        <x:v>Authoritative Week Use</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="F5" s="6" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="G5" s="4"/>
-      <x:c r="H5" s="4"/>
+    <x:row r="5" ht="36" hidden="0" customHeight="1">
+      <x:c r="A5" s="27" t="str">
+        <x:v>Deck #</x:v>
+      </x:c>
+      <x:c r="B5" s="27" t="str">
+        <x:v>Deck Title</x:v>
+      </x:c>
+      <x:c r="C5" s="27" t="str">
+        <x:v>Primary Unit</x:v>
+      </x:c>
+      <x:c r="D5" s="27" t="str">
+        <x:v>Primary Use</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="str">
+        <x:v>Preview / Revisit / Reference Use</x:v>
+      </x:c>
+      <x:c r="F5" s="27" t="str">
+        <x:v>Required Materials by Week</x:v>
+      </x:c>
+      <x:c r="G5" s="27" t="str">
+        <x:v>Optional / Teacher Reference</x:v>
+      </x:c>
+      <x:c r="H5" s="27" t="str">
+        <x:v>Instructional Purpose</x:v>
+      </x:c>
       <x:c r="I5" s="4"/>
       <x:c r="J5" s="4"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="7">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D6" s="16" t="str">
-        <x:v>Primary - Week 1</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="str">
+      <x:c r="A6" s="59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>Authentic Research Course Launch</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>Unit 1</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="str">
+        <x:v>Week 1</x:v>
+      </x:c>
+      <x:c r="E6" s="45" t="str"/>
+      <x:c r="F6" s="45" t="str">
         <x:v>Week 1: U1 H1-H4; U1 Apps A-C</x:v>
       </x:c>
-      <x:c r="F6" s="7" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="G6" s="4"/>
-      <x:c r="H6" s="4"/>
+      <x:c r="G6" s="46" t="str">
+        <x:v>Week 1: U1 Apps I, J, and L</x:v>
+      </x:c>
+      <x:c r="H6" s="62" t="str">
+        <x:v>Course launch and STARLAB identity</x:v>
+      </x:c>
       <x:c r="I6" s="4"/>
       <x:c r="J6" s="4"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="7">
-        <x:v>2.0</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="s">
-        <x:v>164</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D7" s="16" t="str">
-        <x:v>Primary - Week 2</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="str">
+      <x:c r="A7" s="60" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="49" t="str">
+        <x:v>From Topic to Research Question</x:v>
+      </x:c>
+      <x:c r="C7" s="49" t="str">
+        <x:v>Unit 1</x:v>
+      </x:c>
+      <x:c r="D7" s="49" t="str">
+        <x:v>Week 2</x:v>
+      </x:c>
+      <x:c r="E7" s="49" t="str"/>
+      <x:c r="F7" s="49" t="str">
         <x:v>Week 2: U1 H5-H8; U1 Apps D-H</x:v>
       </x:c>
-      <x:c r="F7" s="7" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="G7" s="4"/>
-      <x:c r="H7" s="4"/>
+      <x:c r="G7" s="50" t="str">
+        <x:v>Week 2: U1 Apps I and K</x:v>
+      </x:c>
+      <x:c r="H7" s="63" t="str">
+        <x:v>Topic narrowing and question quality</x:v>
+      </x:c>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
     </x:row>
-    <x:row r="8" ht="24" hidden="0" customHeight="1">
-      <x:c r="A8" s="7">
-        <x:v>3.0</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="D8" s="16" t="str">
-        <x:v>Primary - Week 1; Revisit / Reference - Week 4</x:v>
-      </x:c>
-      <x:c r="E8" s="7" t="str">
-        <x:v>Week 1: U1 H1-H4; U1 Apps A-C; Week 4: U2 H6-H13; U2 Apps E-H</x:v>
-      </x:c>
-      <x:c r="F8" s="7" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="G8" s="4"/>
-      <x:c r="H8" s="4"/>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="61" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="53" t="str">
+        <x:v>Research Ethics, Safety, and Integrity</x:v>
+      </x:c>
+      <x:c r="C8" s="53" t="str">
+        <x:v>Unit 1 / Unit 2</x:v>
+      </x:c>
+      <x:c r="D8" s="53" t="str">
+        <x:v>Week 1</x:v>
+      </x:c>
+      <x:c r="E8" s="53" t="str">
+        <x:v>Revisit / Reference - Week 4</x:v>
+      </x:c>
+      <x:c r="F8" s="53" t="str">
+        <x:v>Week 1: U1 H1-H4; U1 Apps A-C
+Week 4: U2 H6-H13; U2 Apps E-H</x:v>
+      </x:c>
+      <x:c r="G8" s="54" t="str">
+        <x:v>Week 1: U1 Apps I, J, and L
+Week 4: U2 Apps I, J, and L; district forms</x:v>
+      </x:c>
+      <x:c r="H8" s="64" t="str">
+        <x:v>Ethics, safety, and approval culture</x:v>
+      </x:c>
       <x:c r="I8" s="4"/>
       <x:c r="J8" s="4"/>
     </x:row>
-    <x:row r="9" ht="24" hidden="0" customHeight="1">
-      <x:c r="A9" s="7">
-        <x:v>4.0</x:v>
-      </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>169</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="D9" s="16" t="str">
-        <x:v>Primary - Week 2; Revisit / Reference - Week 3</x:v>
-      </x:c>
-      <x:c r="E9" s="7" t="str">
-        <x:v>Week 2: U1 H5-H8; U1 Apps D-H; Week 3: U2 H1-H5; U2 Apps A-D</x:v>
-      </x:c>
-      <x:c r="F9" s="7" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="G9" s="4"/>
-      <x:c r="H9" s="4"/>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="60" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="49" t="str">
+        <x:v>Experimental &amp; Engineering Design Basics</x:v>
+      </x:c>
+      <x:c r="C9" s="49" t="str">
+        <x:v>Unit 1 / Unit 2</x:v>
+      </x:c>
+      <x:c r="D9" s="49" t="str">
+        <x:v>Week 2</x:v>
+      </x:c>
+      <x:c r="E9" s="49" t="str">
+        <x:v>Revisit / Reference - Week 3</x:v>
+      </x:c>
+      <x:c r="F9" s="49" t="str">
+        <x:v>Week 2: U1 H5-H8; U1 Apps D-H
+Week 3: U2 H1-H5; U2 Apps A-D</x:v>
+      </x:c>
+      <x:c r="G9" s="50" t="str">
+        <x:v>Week 2: U1 Apps I and K
+Week 3: U2 App K</x:v>
+      </x:c>
+      <x:c r="H9" s="63" t="str">
+        <x:v>Variables, controls, criteria, constraints</x:v>
+      </x:c>
       <x:c r="I9" s="4"/>
       <x:c r="J9" s="4"/>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="7">
-        <x:v>5.0</x:v>
-      </x:c>
-      <x:c r="B10" s="7" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="D10" s="16" t="str">
-        <x:v>Primary - Weeks 3-4</x:v>
-      </x:c>
-      <x:c r="E10" s="7" t="str">
-        <x:v>Week 3: U2 H1-H5; U2 Apps A-D; Week 4: U2 H6-H13; U2 Apps E-H</x:v>
-      </x:c>
-      <x:c r="F10" s="7" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="G10" s="4"/>
-      <x:c r="H10" s="4"/>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="61" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="53" t="str">
+        <x:v>Building a Formal Research Plan</x:v>
+      </x:c>
+      <x:c r="C10" s="53" t="str">
+        <x:v>Unit 2</x:v>
+      </x:c>
+      <x:c r="D10" s="53" t="str">
+        <x:v>Weeks 3-4</x:v>
+      </x:c>
+      <x:c r="E10" s="53" t="str"/>
+      <x:c r="F10" s="53" t="str">
+        <x:v>Week 3: U2 H1-H5; U2 Apps A-D
+Week 4: U2 H6-H13; U2 Apps E-H</x:v>
+      </x:c>
+      <x:c r="G10" s="54" t="str">
+        <x:v>Week 3: U2 App K
+Week 4: U2 Apps I, J, and L; district forms</x:v>
+      </x:c>
+      <x:c r="H10" s="64" t="str">
+        <x:v>Formal research planning and approval</x:v>
+      </x:c>
       <x:c r="I10" s="4"/>
       <x:c r="J10" s="4"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="7">
-        <x:v>6.0</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="D11" s="16" t="str">
-        <x:v>Primary - Week 5</x:v>
-      </x:c>
-      <x:c r="E11" s="7" t="str">
+      <x:c r="A11" s="60" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="49" t="str">
+        <x:v>Pilot Testing</x:v>
+      </x:c>
+      <x:c r="C11" s="49" t="str">
+        <x:v>Unit 3</x:v>
+      </x:c>
+      <x:c r="D11" s="49" t="str">
+        <x:v>Week 5</x:v>
+      </x:c>
+      <x:c r="E11" s="49" t="str"/>
+      <x:c r="F11" s="49" t="str">
         <x:v>Week 5: U3 H1-H3; U3 Apps A-C</x:v>
       </x:c>
-      <x:c r="F11" s="7" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="G11" s="4"/>
-      <x:c r="H11" s="4"/>
+      <x:c r="G11" s="50" t="str"/>
+      <x:c r="H11" s="63" t="str">
+        <x:v>Testing small before full data collection</x:v>
+      </x:c>
       <x:c r="I11" s="4"/>
       <x:c r="J11" s="4"/>
     </x:row>
-    <x:row r="12" ht="48" hidden="0" customHeight="1">
-      <x:c r="A12" s="7">
-        <x:v>7.0</x:v>
-      </x:c>
-      <x:c r="B12" s="7" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="D12" s="16" t="str">
-        <x:v>Primary - Week 5; ongoing routine reference in Unit 3 (not a scheduled weekly deck)</x:v>
-      </x:c>
-      <x:c r="E12" s="7" t="str">
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="61" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B12" s="53" t="str">
+        <x:v>Research Journals and Documentation</x:v>
+      </x:c>
+      <x:c r="C12" s="53" t="str">
+        <x:v>Unit 3</x:v>
+      </x:c>
+      <x:c r="D12" s="53" t="str">
+        <x:v>Week 5</x:v>
+      </x:c>
+      <x:c r="E12" s="53" t="str">
+        <x:v>Ongoing Unit 3 routine reference (not a separately scheduled weekly deck)</x:v>
+      </x:c>
+      <x:c r="F12" s="53" t="str">
         <x:v>Week 5: U3 H1-H3; U3 Apps A-C</x:v>
       </x:c>
-      <x:c r="F12" s="7" t="s">
-        <x:v>176</x:v>
-      </x:c>
-      <x:c r="G12" s="4"/>
-      <x:c r="H12" s="4"/>
+      <x:c r="G12" s="54" t="str"/>
+      <x:c r="H12" s="64" t="str">
+        <x:v>Journal setup and scientific documentation</x:v>
+      </x:c>
       <x:c r="I12" s="4"/>
       <x:c r="J12" s="4"/>
     </x:row>
-    <x:row r="13" ht="36" hidden="0" customHeight="1">
-      <x:c r="A13" s="7">
-        <x:v>8.0</x:v>
-      </x:c>
-      <x:c r="B13" s="7" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="D13" s="16" t="str">
-        <x:v>Primary - Week 6; Revisit / Reference - Weeks 7, 10, and 13</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="str">
-        <x:v>Week 6: U3 H4-H5; U3 Apps D-E; Week 7: U3 H6-H7; U3 Apps F-G; Week 10: U3 H11-H12; Week 13: U3 H9, H15</x:v>
-      </x:c>
-      <x:c r="F13" s="7" t="s">
-        <x:v>178</x:v>
-      </x:c>
-      <x:c r="G13" s="4"/>
-      <x:c r="H13" s="4"/>
+    <x:row r="13" ht="48" hidden="0" customHeight="1">
+      <x:c r="A13" s="60" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B13" s="49" t="str">
+        <x:v>Troubleshooting and Responsible Project Pivots</x:v>
+      </x:c>
+      <x:c r="C13" s="49" t="str">
+        <x:v>Unit 3</x:v>
+      </x:c>
+      <x:c r="D13" s="49" t="str">
+        <x:v>Week 6</x:v>
+      </x:c>
+      <x:c r="E13" s="49" t="str">
+        <x:v>Revisit / Reference - Weeks 7, 10, and 13</x:v>
+      </x:c>
+      <x:c r="F13" s="49" t="str">
+        <x:v>Week 6: U3 H4-H5; U3 Apps D-E
+Week 7: U3 H6-H7; U3 Apps F-G
+Week 10: U3 H11-H12
+Week 13: U3 H9 and H15</x:v>
+      </x:c>
+      <x:c r="G13" s="50" t="str">
+        <x:v>Week 10: U3 Apps K-L
+Week 13: U3 App P</x:v>
+      </x:c>
+      <x:c r="H13" s="63" t="str">
+        <x:v>Diagnose, revise, document, pivot responsibly</x:v>
+      </x:c>
       <x:c r="I13" s="4"/>
       <x:c r="J13" s="4"/>
     </x:row>
-    <x:row r="14" ht="36" hidden="0" customHeight="1">
-      <x:c r="A14" s="7">
-        <x:v>9.0</x:v>
-      </x:c>
-      <x:c r="B14" s="7" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="D14" s="16" t="str">
-        <x:v>Primary - Weeks 15 and 17; Revisit / Reference - Weeks 9 and 16</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="str">
-        <x:v>Week 9: U3 H9-H10; Week 15: U3 H17; U3 Apps Q-R; Week 16: U3 H18-H19; Week 17: U4 H1-H4; U4 Apps A-C</x:v>
-      </x:c>
-      <x:c r="F14" s="7" t="s">
-        <x:v>181</x:v>
-      </x:c>
-      <x:c r="G14" s="4"/>
-      <x:c r="H14" s="4"/>
+    <x:row r="14" ht="48" hidden="0" customHeight="1">
+      <x:c r="A14" s="61" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B14" s="53" t="str">
+        <x:v>Data Organization: Raw Data vs. Clean Data</x:v>
+      </x:c>
+      <x:c r="C14" s="53" t="str">
+        <x:v>Unit 3 / Unit 4</x:v>
+      </x:c>
+      <x:c r="D14" s="53" t="str">
+        <x:v>Weeks 15 and 17</x:v>
+      </x:c>
+      <x:c r="E14" s="53" t="str">
+        <x:v>Revisit / Reference - Weeks 9 and 16</x:v>
+      </x:c>
+      <x:c r="F14" s="53" t="str">
+        <x:v>Week 9: U3 H9-H10
+Week 15: U3 H17; U3 Apps Q-R
+Week 16: U3 H18-H19
+Week 17: U4 H1-H4; U4 Apps A-C</x:v>
+      </x:c>
+      <x:c r="G14" s="54" t="str">
+        <x:v>Week 9: U3 App J
+Week 16: U3 Apps S-U</x:v>
+      </x:c>
+      <x:c r="H14" s="64" t="str">
+        <x:v>Preserve raw data and create clean copies</x:v>
+      </x:c>
       <x:c r="I14" s="4"/>
       <x:c r="J14" s="4"/>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="7">
-        <x:v>10.0</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="D15" s="16" t="str">
-        <x:v>Primary - Weeks 17-18</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="str">
-        <x:v>Week 17: U4 H1-H4; U4 Apps A-C; Week 18: U4 H5-H8; U4 Apps D-G</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="G15" s="4"/>
-      <x:c r="H15" s="4"/>
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
+      <x:c r="A15" s="60" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B15" s="49" t="str">
+        <x:v>Choosing the Right Data Analysis Method</x:v>
+      </x:c>
+      <x:c r="C15" s="49" t="str">
+        <x:v>Unit 4</x:v>
+      </x:c>
+      <x:c r="D15" s="49" t="str">
+        <x:v>Weeks 17-18</x:v>
+      </x:c>
+      <x:c r="E15" s="49" t="str"/>
+      <x:c r="F15" s="49" t="str">
+        <x:v>Week 17: U4 H1-H4; U4 Apps A-C
+Week 18: U4 H5-H8; U4 Apps D-G</x:v>
+      </x:c>
+      <x:c r="G15" s="50" t="str"/>
+      <x:c r="H15" s="63" t="str">
+        <x:v>Match data type to analysis method</x:v>
+      </x:c>
       <x:c r="I15" s="4"/>
       <x:c r="J15" s="4"/>
     </x:row>
     <x:row r="16" ht="24" hidden="0" customHeight="1">
-      <x:c r="A16" s="7">
-        <x:v>11.0</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="s">
-        <x:v>184</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="D16" s="16" t="str">
-        <x:v>Primary - Week 19; Revisit / Reference - Week 24</x:v>
-      </x:c>
-      <x:c r="E16" s="7" t="str">
-        <x:v>Week 19: U4 H9-H12; U4 Apps H-K; Week 24: U5 H5; U5 Apps F-G</x:v>
-      </x:c>
-      <x:c r="F16" s="7" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="G16" s="4"/>
-      <x:c r="H16" s="4"/>
+      <x:c r="A16" s="61" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B16" s="53" t="str">
+        <x:v>Graphing and Visual Ethics</x:v>
+      </x:c>
+      <x:c r="C16" s="53" t="str">
+        <x:v>Unit 4 / Unit 5</x:v>
+      </x:c>
+      <x:c r="D16" s="53" t="str">
+        <x:v>Week 19</x:v>
+      </x:c>
+      <x:c r="E16" s="53" t="str">
+        <x:v>Revisit / Reference - Week 24</x:v>
+      </x:c>
+      <x:c r="F16" s="53" t="str">
+        <x:v>Week 19: U4 H9-H12; U4 Apps H-K
+Week 24: U5 H5; U5 Apps F-G</x:v>
+      </x:c>
+      <x:c r="G16" s="54" t="str"/>
+      <x:c r="H16" s="64" t="str">
+        <x:v>Clear, honest data visuals</x:v>
+      </x:c>
       <x:c r="I16" s="4"/>
       <x:c r="J16" s="4"/>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
-      <x:c r="A17" s="7">
-        <x:v>12.0</x:v>
-      </x:c>
-      <x:c r="B17" s="7" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="D17" s="16" t="str">
-        <x:v>Primary - Week 19; Revisit / Reference - Week 20</x:v>
-      </x:c>
-      <x:c r="E17" s="7" t="str">
-        <x:v>Week 19: U4 H9-H12; U4 Apps H-K; Week 20: U4 H13-H17; U4 App N</x:v>
-      </x:c>
-      <x:c r="F17" s="7" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="G17" s="4"/>
-      <x:c r="H17" s="4"/>
+      <x:c r="A17" s="60" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B17" s="49" t="str">
+        <x:v>Error, Uncertainty, and Limitations</x:v>
+      </x:c>
+      <x:c r="C17" s="49" t="str">
+        <x:v>Unit 4</x:v>
+      </x:c>
+      <x:c r="D17" s="49" t="str">
+        <x:v>Week 19</x:v>
+      </x:c>
+      <x:c r="E17" s="49" t="str">
+        <x:v>Revisit / Reference - Week 20</x:v>
+      </x:c>
+      <x:c r="F17" s="49" t="str">
+        <x:v>Week 19: U4 H9-H12; U4 Apps H-K
+Week 20: U4 H13-H17; U4 App N</x:v>
+      </x:c>
+      <x:c r="G17" s="50" t="str">
+        <x:v>Week 20: U4 Apps L-M and O-Q</x:v>
+      </x:c>
+      <x:c r="H17" s="63" t="str">
+        <x:v>Interpret evidence with caution</x:v>
+      </x:c>
       <x:c r="I17" s="4"/>
       <x:c r="J17" s="4"/>
     </x:row>
-    <x:row r="18" ht="36" hidden="0" customHeight="1">
-      <x:c r="A18" s="7">
-        <x:v>13.0</x:v>
-      </x:c>
-      <x:c r="B18" s="7" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D18" s="16" t="str">
-        <x:v>Primary - Week 21; Revisit / Reference - Weeks 22, 23, and 26</x:v>
-      </x:c>
-      <x:c r="E18" s="7" t="str">
-        <x:v>Week 21: U5 H1-H2; U5 Apps A, L; Week 22: U5 H3; U5 Apps B-C; Week 23: U5 H4; U5 Apps D-E; Week 26: U5 H7; U5 Apps J-L</x:v>
-      </x:c>
-      <x:c r="F18" s="7" t="s">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="G18" s="4"/>
-      <x:c r="H18" s="4"/>
+    <x:row r="18" ht="48" hidden="0" customHeight="1">
+      <x:c r="A18" s="61" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B18" s="53" t="str">
+        <x:v>Scientific Report Structure</x:v>
+      </x:c>
+      <x:c r="C18" s="53" t="str">
+        <x:v>Unit 5</x:v>
+      </x:c>
+      <x:c r="D18" s="53" t="str">
+        <x:v>Week 21</x:v>
+      </x:c>
+      <x:c r="E18" s="53" t="str">
+        <x:v>Revisit / Reference - Weeks 22, 23, and 26</x:v>
+      </x:c>
+      <x:c r="F18" s="53" t="str">
+        <x:v>Week 21: U5 H1-H2; U5 Apps A and L
+Week 22: U5 H3; U5 Apps B-C
+Week 23: U5 H4; U5 Apps D-E
+Week 26: U5 H7; U5 Apps J-L</x:v>
+      </x:c>
+      <x:c r="G18" s="54" t="str">
+        <x:v>Week 21: U5 Apps R-S</x:v>
+      </x:c>
+      <x:c r="H18" s="64" t="str">
+        <x:v>Report architecture and planning</x:v>
+      </x:c>
       <x:c r="I18" s="4"/>
       <x:c r="J18" s="4"/>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="7">
-        <x:v>14.0</x:v>
-      </x:c>
-      <x:c r="B19" s="7" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D19" s="16" t="str">
-        <x:v>Primary - Week 25</x:v>
-      </x:c>
-      <x:c r="E19" s="7" t="str">
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="60" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B19" s="49" t="str">
+        <x:v>Writing the Discussion: CER</x:v>
+      </x:c>
+      <x:c r="C19" s="49" t="str">
+        <x:v>Unit 5</x:v>
+      </x:c>
+      <x:c r="D19" s="49" t="str">
+        <x:v>Week 25</x:v>
+      </x:c>
+      <x:c r="E19" s="49" t="str"/>
+      <x:c r="F19" s="49" t="str">
         <x:v>Week 25: U5 H6; U5 Apps H-I</x:v>
       </x:c>
-      <x:c r="F19" s="7" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="G19" s="4"/>
-      <x:c r="H19" s="4"/>
+      <x:c r="G19" s="50" t="str"/>
+      <x:c r="H19" s="63" t="str">
+        <x:v>Claim-evidence-reasoning, limitations, future work</x:v>
+      </x:c>
       <x:c r="I19" s="4"/>
       <x:c r="J19" s="4"/>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="7">
-        <x:v>15.0</x:v>
-      </x:c>
-      <x:c r="B20" s="7" t="s">
-        <x:v>193</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D20" s="16" t="str">
-        <x:v>Primary - Week 27</x:v>
-      </x:c>
-      <x:c r="E20" s="7" t="str">
+      <x:c r="A20" s="61" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B20" s="53" t="str">
+        <x:v>Peer Review and Scientific Revision</x:v>
+      </x:c>
+      <x:c r="C20" s="53" t="str">
+        <x:v>Unit 5</x:v>
+      </x:c>
+      <x:c r="D20" s="53" t="str">
+        <x:v>Week 27</x:v>
+      </x:c>
+      <x:c r="E20" s="53" t="str"/>
+      <x:c r="F20" s="53" t="str">
         <x:v>Week 27: U5 H8-H9; U5 Apps M-N</x:v>
       </x:c>
-      <x:c r="F20" s="7" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="G20" s="4"/>
-      <x:c r="H20" s="4"/>
+      <x:c r="G20" s="54" t="str">
+        <x:v>Previously issued reference: U5 Apps J-L</x:v>
+      </x:c>
+      <x:c r="H20" s="64" t="str">
+        <x:v>Structured feedback and revision</x:v>
+      </x:c>
       <x:c r="I20" s="4"/>
       <x:c r="J20" s="4"/>
     </x:row>
-    <x:row r="21" ht="24" hidden="0" customHeight="1">
-      <x:c r="A21" s="7">
-        <x:v>16.0</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="s">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="D21" s="16" t="str">
-        <x:v>Primary - Week 28; Revisit / Reference - Week 32</x:v>
-      </x:c>
-      <x:c r="E21" s="7" t="str">
-        <x:v>Week 28: U5 H10-H11; U5 App O; Week 32: U6 H10-H12</x:v>
-      </x:c>
-      <x:c r="F21" s="7" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="G21" s="4"/>
-      <x:c r="H21" s="4"/>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="60" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B21" s="49" t="str">
+        <x:v>Designing a Research Poster or Presentation Board</x:v>
+      </x:c>
+      <x:c r="C21" s="49" t="str">
+        <x:v>Unit 5 / Unit 6</x:v>
+      </x:c>
+      <x:c r="D21" s="49" t="str">
+        <x:v>Week 28</x:v>
+      </x:c>
+      <x:c r="E21" s="49" t="str">
+        <x:v>Revisit / Reference - Week 32</x:v>
+      </x:c>
+      <x:c r="F21" s="49" t="str">
+        <x:v>Week 28: U5 H10-H11; U5 App O
+Week 32: U6 H10-H12</x:v>
+      </x:c>
+      <x:c r="G21" s="50" t="str">
+        <x:v>Week 28: U5 App Q
+Week 32: U6 Apps I-L</x:v>
+      </x:c>
+      <x:c r="H21" s="63" t="str">
+        <x:v>Visual aid and showcase preparation</x:v>
+      </x:c>
       <x:c r="I21" s="4"/>
       <x:c r="J21" s="4"/>
     </x:row>
-    <x:row r="22" ht="48" hidden="0" customHeight="1">
-      <x:c r="A22" s="7">
-        <x:v>17.0</x:v>
-      </x:c>
-      <x:c r="B22" s="7" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="D22" s="16" t="str">
-        <x:v>Preview / Reference - Week 28; Primary - Week 29; Revisit / Reference - Week 30</x:v>
-      </x:c>
-      <x:c r="E22" s="7" t="str">
-        <x:v>Week 28: U5 H10-H11; U5 App O; Weeks 29-30: U6 H1-H6; U6 Apps A-E</x:v>
-      </x:c>
-      <x:c r="F22" s="7" t="s">
-        <x:v>199</x:v>
-      </x:c>
-      <x:c r="G22" s="4"/>
-      <x:c r="H22" s="4"/>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A22" s="61" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B22" s="53" t="str">
+        <x:v>Oral Presentation Skills for Research</x:v>
+      </x:c>
+      <x:c r="C22" s="53" t="str">
+        <x:v>Unit 6</x:v>
+      </x:c>
+      <x:c r="D22" s="53" t="str">
+        <x:v>Week 29</x:v>
+      </x:c>
+      <x:c r="E22" s="53" t="str">
+        <x:v>Preview / Reference - Week 28
+Revisit / Reference - Week 30</x:v>
+      </x:c>
+      <x:c r="F22" s="53" t="str">
+        <x:v>Week 28: U5 H10-H11; U5 App O
+Weeks 29-30: U6 H1-H6; U6 Apps A-E</x:v>
+      </x:c>
+      <x:c r="G22" s="54" t="str">
+        <x:v>Weeks 28-30: U6 App L
+Week 28: U5 App Q</x:v>
+      </x:c>
+      <x:c r="H22" s="64" t="str">
+        <x:v>Research story, speaking notes, practice</x:v>
+      </x:c>
       <x:c r="I22" s="4"/>
       <x:c r="J22" s="4"/>
     </x:row>
-    <x:row r="23" ht="24" hidden="0" customHeight="1">
-      <x:c r="A23" s="7">
-        <x:v>18.0</x:v>
-      </x:c>
-      <x:c r="B23" s="7" t="s">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="D23" s="16" t="str">
-        <x:v>Primary - Week 31; Revisit / Reference - Week 32</x:v>
-      </x:c>
-      <x:c r="E23" s="7" t="str">
-        <x:v>Week 31: U6 H7-H9; U6 Apps F-H; Week 32: U6 H10-H12</x:v>
-      </x:c>
-      <x:c r="F23" s="7" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="G23" s="4"/>
-      <x:c r="H23" s="4"/>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A23" s="60" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B23" s="49" t="str">
+        <x:v>Answering Questions Like a Scientist</x:v>
+      </x:c>
+      <x:c r="C23" s="49" t="str">
+        <x:v>Unit 6</x:v>
+      </x:c>
+      <x:c r="D23" s="49" t="str">
+        <x:v>Week 31</x:v>
+      </x:c>
+      <x:c r="E23" s="49" t="str">
+        <x:v>Revisit / Reference - Week 32</x:v>
+      </x:c>
+      <x:c r="F23" s="49" t="str">
+        <x:v>Week 31: U6 H7-H9; U6 Apps F-H
+Week 32: U6 H10-H12</x:v>
+      </x:c>
+      <x:c r="G23" s="50" t="str">
+        <x:v>Weeks 31-32: U6 App L
+Week 32: U6 Apps I-K</x:v>
+      </x:c>
+      <x:c r="H23" s="63" t="str">
+        <x:v>Q&amp;A, evidence defense, scientific humility</x:v>
+      </x:c>
       <x:c r="I23" s="4"/>
       <x:c r="J23" s="4"/>
     </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="7">
-        <x:v>19.0</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C24" s="7" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="D24" s="16" t="str">
-        <x:v>Primary - Week 34</x:v>
-      </x:c>
-      <x:c r="E24" s="7" t="str">
-        <x:v>Week 34: U6 H15-H16, H18</x:v>
-      </x:c>
-      <x:c r="F24" s="7" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="G24" s="4"/>
-      <x:c r="H24" s="4"/>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A24" s="61" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B24" s="53" t="str">
+        <x:v>Final Reflection and Research Portfolio</x:v>
+      </x:c>
+      <x:c r="C24" s="53" t="str">
+        <x:v>Unit 6</x:v>
+      </x:c>
+      <x:c r="D24" s="53" t="str">
+        <x:v>Week 34</x:v>
+      </x:c>
+      <x:c r="E24" s="53" t="str"/>
+      <x:c r="F24" s="53" t="str">
+        <x:v>Week 34: U6 H15-H16 and H18</x:v>
+      </x:c>
+      <x:c r="G24" s="54" t="str">
+        <x:v>Week 34: U6 H17; U6 Apps O-S</x:v>
+      </x:c>
+      <x:c r="H24" s="64" t="str">
+        <x:v>Portfolio, reflection, continuation planning</x:v>
+      </x:c>
       <x:c r="I24" s="4"/>
       <x:c r="J24" s="4"/>
     </x:row>
@@ -7925,7 +8188,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fbf688b67b543f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdd4af4819784406"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7945,12 +8208,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>204</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>205</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -7976,16 +8239,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>206</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
-        <x:v>208</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="F5" s="6" t="s">
-        <x:v>209</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
@@ -9892,7 +10155,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redb8c45a072448ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5044cccf93447d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9910,12 +10173,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>210</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>211</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -9935,16 +10198,16 @@
     </x:row>
     <x:row r="5" ht="31.5" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>212</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>213</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>214</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
         <x:v>9</x:v>
@@ -9957,16 +10220,16 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="s">
-        <x:v>216</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
-        <x:v>217</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="E6" s="7" t="s">
         <x:v>15</x:v>
@@ -9979,16 +10242,16 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7" t="s">
-        <x:v>220</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="C7" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D7" s="7" t="s">
-        <x:v>223</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="E7" s="7" t="s">
         <x:v>15</x:v>
@@ -10001,10 +10264,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7" t="s">
-        <x:v>224</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
-        <x:v>225</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
         <x:v>Students hold an exact Project Approval Tracker status and have concrete next steps</x:v>
@@ -10023,16 +10286,16 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7" t="s">
-        <x:v>226</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
-        <x:v>227</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>228</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D9" s="7" t="s">
-        <x:v>229</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="E9" s="7" t="s">
         <x:v>27</x:v>
@@ -10045,16 +10308,16 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7" t="s">
-        <x:v>230</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B10" s="7" t="s">
-        <x:v>231</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
         <x:v>Students revise, retest, or receive Approved for Systematic Data Collection in the tracker</x:v>
       </x:c>
       <x:c r="D10" s="7" t="s">
-        <x:v>232</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E10" s="7" t="s">
         <x:v>27</x:v>
@@ -10067,13 +10330,13 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7" t="s">
-        <x:v>233</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
-        <x:v>234</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="C11" s="7" t="s">
-        <x:v>235</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="D11" s="7" t="str">
         <x:v>Record Approved for Systematic Data Collection before full collection begins</x:v>
@@ -10089,16 +10352,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7" t="s">
-        <x:v>236</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B12" s="7" t="s">
-        <x:v>237</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="C12" s="7" t="s">
-        <x:v>238</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="D12" s="7" t="s">
-        <x:v>239</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="E12" s="7" t="s">
         <x:v>27</x:v>
@@ -10111,16 +10374,16 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="B13" s="7" t="s">
-        <x:v>241</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C13" s="7" t="s">
-        <x:v>242</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D13" s="7" t="s">
-        <x:v>243</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E13" s="7" t="s">
         <x:v>27</x:v>
@@ -10133,16 +10396,16 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7" t="s">
-        <x:v>244</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B14" s="7" t="s">
-        <x:v>245</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C14" s="7" t="s">
-        <x:v>246</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="D14" s="7" t="s">
-        <x:v>247</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="E14" s="7" t="s">
         <x:v>33</x:v>
@@ -10155,16 +10418,16 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7" t="s">
-        <x:v>248</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B15" s="7" t="s">
-        <x:v>249</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C15" s="7" t="s">
-        <x:v>250</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D15" s="7" t="s">
-        <x:v>251</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="E15" s="7" t="s">
         <x:v>33</x:v>
@@ -10177,16 +10440,16 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7" t="s">
-        <x:v>252</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="B16" s="7" t="s">
-        <x:v>253</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="C16" s="7" t="s">
-        <x:v>254</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D16" s="7" t="s">
-        <x:v>255</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E16" s="7" t="s">
         <x:v>33</x:v>
@@ -10199,16 +10462,16 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7" t="s">
-        <x:v>256</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
-        <x:v>257</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="C17" s="7" t="s">
-        <x:v>258</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="D17" s="7" t="s">
-        <x:v>259</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="E17" s="7" t="s">
         <x:v>33</x:v>
@@ -10221,13 +10484,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="7" t="s">
-        <x:v>260</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
         <x:v>Report and public showcase planning launch</x:v>
       </x:c>
       <x:c r="C18" s="7" t="s">
-        <x:v>261</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
         <x:v>Set public format, target date, audience, and space six to eight weeks ahead</x:v>
@@ -10243,16 +10506,16 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="7" t="s">
-        <x:v>262</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="B19" s="7" t="s">
-        <x:v>263</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="C19" s="7" t="s">
-        <x:v>264</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="D19" s="7" t="s">
-        <x:v>265</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="E19" s="7" t="s">
         <x:v>39</x:v>
@@ -10265,16 +10528,16 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="7" t="s">
-        <x:v>266</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B20" s="7" t="s">
-        <x:v>267</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="C20" s="7" t="s">
-        <x:v>268</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
-        <x:v>269</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="E20" s="7" t="s">
         <x:v>39</x:v>
@@ -10287,13 +10550,13 @@
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="7" t="s">
-        <x:v>270</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B21" s="7" t="str">
         <x:v>Presentation product and event readiness</x:v>
       </x:c>
       <x:c r="C21" s="7" t="s">
-        <x:v>271</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="D21" s="7" t="str">
         <x:v>Check readability and presentation story; finalize public event logistics</x:v>
@@ -10309,16 +10572,16 @@
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
       <x:c r="A22" s="7" t="s">
-        <x:v>272</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B22" s="7" t="s">
-        <x:v>273</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="C22" s="7" t="s">
-        <x:v>274</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="D22" s="7" t="s">
-        <x:v>275</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="E22" s="7" t="s">
         <x:v>45</x:v>
@@ -10331,16 +10594,16 @@
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="7" t="s">
-        <x:v>276</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="B23" s="7" t="s">
-        <x:v>277</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C23" s="7" t="s">
-        <x:v>278</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="D23" s="7" t="s">
-        <x:v>279</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="E23" s="7" t="s">
         <x:v>45</x:v>
@@ -10353,7 +10616,7 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="7" t="s">
-        <x:v>280</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
         <x:v>Required public presentation/showcase</x:v>
@@ -10375,16 +10638,16 @@
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="7" t="s">
-        <x:v>281</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="B25" s="7" t="s">
-        <x:v>282</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C25" s="7" t="s">
-        <x:v>283</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="D25" s="7" t="s">
-        <x:v>284</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="E25" s="7" t="s">
         <x:v>45</x:v>
@@ -11983,7 +12246,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6547a95374e14ddf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae3c4313a7248c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12003,12 +12266,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>285</x:v>
+        <x:v>238</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>286</x:v>
+        <x:v>239</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -12037,13 +12300,13 @@
         <x:v>Deck Use</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>287</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="F5" s="6" t="s">
-        <x:v>289</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
@@ -12063,7 +12326,9 @@
       <x:c r="D6" s="7" t="str">
         <x:v>U1 H1; U1 H2; U1 H3; U1 H4; U1 App A; U1 App B; U1 App C</x:v>
       </x:c>
-      <x:c r="E6" s="7" t="str"/>
+      <x:c r="E6" s="7" t="str">
+        <x:v>U1 App I; U1 App J; U1 App L</x:v>
+      </x:c>
       <x:c r="F6" s="7" t="s">
         <x:v>60</x:v>
       </x:c>
@@ -12086,7 +12351,7 @@
         <x:v>U1 H5; U1 H6; U1 H7; U1 H8; U1 App D; U1 App E; U1 App F; U1 App G; U1 App H</x:v>
       </x:c>
       <x:c r="E7" s="7" t="str">
-        <x:v>U1 App I</x:v>
+        <x:v>U1 App I; U1 App K</x:v>
       </x:c>
       <x:c r="F7" s="7" t="s">
         <x:v>63</x:v>
@@ -12109,7 +12374,9 @@
       <x:c r="D8" s="7" t="str">
         <x:v>U2 H1; U2 H2; U2 H3; U2 H4; U2 H5; U2 App A; U2 App B; U2 App C; U2 App D</x:v>
       </x:c>
-      <x:c r="E8" s="7" t="str"/>
+      <x:c r="E8" s="7" t="str">
+        <x:v>U2 App K</x:v>
+      </x:c>
       <x:c r="F8" s="7" t="s">
         <x:v>66</x:v>
       </x:c>
@@ -12132,7 +12399,7 @@
         <x:v>U2 H6; U2 H7; U2 H8; U2 H9; U2 H10; U2 H11; U2 H12; U2 H13; U2 App E; U2 App F; U2 App G; U2 App H</x:v>
       </x:c>
       <x:c r="E9" s="7" t="str">
-        <x:v>U2 AppI; U2 AppJ; district-supplied approval and safety forms as applicable</x:v>
+        <x:v>U2 App I; U2 App J; U2 App L; district-supplied approval and safety forms as applicable</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
         <x:v>69</x:v>
@@ -12155,7 +12422,7 @@
       <x:c r="D10" s="7" t="str">
         <x:v>U3 H1; U3 H2; U3 H3; U3 App A; U3 App B; U3 App C</x:v>
       </x:c>
-      <x:c r="E10" s="7" t="str"/>
+      <x:c r="E10" s="7"/>
       <x:c r="F10" s="7" t="s">
         <x:v>72</x:v>
       </x:c>
@@ -12177,7 +12444,7 @@
       <x:c r="D11" s="7" t="str">
         <x:v>U3 H4; U3 H5; U3 App D; U3 App E</x:v>
       </x:c>
-      <x:c r="E11" s="7" t="str"/>
+      <x:c r="E11" s="7"/>
       <x:c r="F11" s="7" t="s">
         <x:v>75</x:v>
       </x:c>
@@ -12199,7 +12466,7 @@
       <x:c r="D12" s="7" t="str">
         <x:v>U3 H6; U3 H7; U3 App F; U3 App G</x:v>
       </x:c>
-      <x:c r="E12" s="7" t="str"/>
+      <x:c r="E12" s="7"/>
       <x:c r="F12" s="7" t="s">
         <x:v>78</x:v>
       </x:c>
@@ -12365,7 +12632,7 @@
       <x:c r="D19" s="7" t="str">
         <x:v>U3 H9; U3 H16</x:v>
       </x:c>
-      <x:c r="E19" s="7" t="str"/>
+      <x:c r="E19" s="7"/>
       <x:c r="F19" s="7" t="s">
         <x:v>99</x:v>
       </x:c>
@@ -12387,7 +12654,7 @@
       <x:c r="D20" s="7" t="str">
         <x:v>U3 H17; U3 App Q; U3 App R</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="str"/>
+      <x:c r="E20" s="7"/>
       <x:c r="F20" s="7" t="s">
         <x:v>102</x:v>
       </x:c>
@@ -12433,7 +12700,7 @@
       <x:c r="D22" s="7" t="str">
         <x:v>U4 H1; U4 H2; U4 H3; U4 H4; U4 App A; U4 App B; U4 App C</x:v>
       </x:c>
-      <x:c r="E22" s="7" t="str"/>
+      <x:c r="E22" s="7"/>
       <x:c r="F22" s="7" t="s">
         <x:v>108</x:v>
       </x:c>
@@ -12455,7 +12722,7 @@
       <x:c r="D23" s="7" t="str">
         <x:v>U4 H5; U4 H6; U4 H7; U4 H8; U4 App D; U4 App E; U4 App F; U4 App G</x:v>
       </x:c>
-      <x:c r="E23" s="7" t="str"/>
+      <x:c r="E23" s="7"/>
       <x:c r="F23" s="7" t="s">
         <x:v>111</x:v>
       </x:c>
@@ -12477,7 +12744,7 @@
       <x:c r="D24" s="7" t="str">
         <x:v>U4 H9; U4 H10; U4 H11; U4 H12; U4 App H; U4 App I; U4 App J; U4 App K</x:v>
       </x:c>
-      <x:c r="E24" s="7" t="str"/>
+      <x:c r="E24" s="7"/>
       <x:c r="F24" s="7" t="s">
         <x:v>114</x:v>
       </x:c>
@@ -12523,7 +12790,9 @@
       <x:c r="D26" s="7" t="str">
         <x:v>U5 H1; U5 H2; U5 App A; U5 App L</x:v>
       </x:c>
-      <x:c r="E26" s="7" t="str"/>
+      <x:c r="E26" s="7" t="str">
+        <x:v>U5 App R; U5 App S</x:v>
+      </x:c>
       <x:c r="F26" s="7" t="s">
         <x:v>120</x:v>
       </x:c>
@@ -12545,7 +12814,7 @@
       <x:c r="D27" s="7" t="str">
         <x:v>U5 H3; U5 App B; U5 App C</x:v>
       </x:c>
-      <x:c r="E27" s="7" t="str"/>
+      <x:c r="E27" s="7"/>
       <x:c r="F27" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
@@ -12567,7 +12836,7 @@
       <x:c r="D28" s="7" t="str">
         <x:v>U5 H4; U5 App D; U5 App E</x:v>
       </x:c>
-      <x:c r="E28" s="7" t="str"/>
+      <x:c r="E28" s="7"/>
       <x:c r="F28" s="7" t="s">
         <x:v>125</x:v>
       </x:c>
@@ -12589,7 +12858,7 @@
       <x:c r="D29" s="7" t="str">
         <x:v>U5 H5; U5 App F; U5 App G</x:v>
       </x:c>
-      <x:c r="E29" s="7" t="str"/>
+      <x:c r="E29" s="7"/>
       <x:c r="F29" s="7" t="s">
         <x:v>128</x:v>
       </x:c>
@@ -12611,7 +12880,7 @@
       <x:c r="D30" s="7" t="str">
         <x:v>U5 H6; U5 App H; U5 App I</x:v>
       </x:c>
-      <x:c r="E30" s="7" t="str"/>
+      <x:c r="E30" s="7"/>
       <x:c r="F30" s="7" t="s">
         <x:v>130</x:v>
       </x:c>
@@ -12633,7 +12902,7 @@
       <x:c r="D31" s="7" t="str">
         <x:v>U5 H7; U5 App J; U5 App K; U5 App L</x:v>
       </x:c>
-      <x:c r="E31" s="7" t="str"/>
+      <x:c r="E31" s="7"/>
       <x:c r="F31" s="7" t="s">
         <x:v>133</x:v>
       </x:c>
@@ -12655,7 +12924,7 @@
       <x:c r="D32" s="7" t="str">
         <x:v>U5 H8; U5 H9; U5 App M; U5 App N</x:v>
       </x:c>
-      <x:c r="E32" s="7" t="str"/>
+      <x:c r="E32" s="7"/>
       <x:c r="F32" s="7" t="s">
         <x:v>136</x:v>
       </x:c>
@@ -12678,7 +12947,7 @@
         <x:v>U5 H10; U5 H11; U5 App O</x:v>
       </x:c>
       <x:c r="E33" s="7" t="str">
-        <x:v>U5 App Q</x:v>
+        <x:v>U5 App Q; U6 App L</x:v>
       </x:c>
       <x:c r="F33" s="7" t="s">
         <x:v>138</x:v>
@@ -12701,7 +12970,9 @@
       <x:c r="D34" s="7" t="str">
         <x:v>U6 H1; U6 H2; U6 H3; U6 App A; U6 App B; U6 App C</x:v>
       </x:c>
-      <x:c r="E34" s="7" t="str"/>
+      <x:c r="E34" s="7" t="str">
+        <x:v>U6 App L</x:v>
+      </x:c>
       <x:c r="F34" s="7" t="s">
         <x:v>141</x:v>
       </x:c>
@@ -12723,7 +12994,9 @@
       <x:c r="D35" s="7" t="str">
         <x:v>U6 H4; U6 H5; U6 H6; U6 App D; U6 App E</x:v>
       </x:c>
-      <x:c r="E35" s="7" t="str"/>
+      <x:c r="E35" s="7" t="str">
+        <x:v>U6 App L</x:v>
+      </x:c>
       <x:c r="F35" s="7" t="s">
         <x:v>144</x:v>
       </x:c>
@@ -12745,7 +13018,9 @@
       <x:c r="D36" s="7" t="str">
         <x:v>U6 H7; U6 H8; U6 H9; U6 App F; U6 App G; U6 App H</x:v>
       </x:c>
-      <x:c r="E36" s="7" t="str"/>
+      <x:c r="E36" s="7" t="str">
+        <x:v>U6 App L</x:v>
+      </x:c>
       <x:c r="F36" s="7" t="s">
         <x:v>147</x:v>
       </x:c>
@@ -12768,7 +13043,7 @@
         <x:v>U6 H10; U6 H11; U6 H12</x:v>
       </x:c>
       <x:c r="E37" s="7" t="str">
-        <x:v>U6 App I; U6 App J; U6 App K</x:v>
+        <x:v>U6 App I; U6 App J; U6 App K; U6 App L</x:v>
       </x:c>
       <x:c r="F37" s="7" t="s">
         <x:v>150</x:v>
@@ -12795,7 +13070,7 @@
         <x:v>U6 App N</x:v>
       </x:c>
       <x:c r="F38" s="7" t="s">
-        <x:v>290</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="G38" s="4"/>
       <x:c r="H38" s="4"/>
@@ -14246,7 +14521,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67f6c047978e4cbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8209c34c3df467d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add advance showcase planning milestones
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
+++ b/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R65be224c0ae1428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="Rb616e6b4b1944c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="Rdb3db2c035514e58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R10f67599e3954b84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="R2bb4c2568c174fe4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="R8eb035c0a96f4dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R33580968ffa4498f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="R004d08fdd2d84867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="R37485dac14564475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R06669ac9983f4136"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="Rda452686af514614"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="R01fd915949cc4b57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -378,9 +378,6 @@
     <x:t xml:space="preserve">Annotated model report, strong/weak comparison, report planning map</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">This week is architecture, not polished writing</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Introduction planning organizer, introduction draft, peer feedback</x:t>
   </x:si>
   <x:si>
@@ -402,9 +399,6 @@
     <x:t xml:space="preserve">Final/near-final visuals, captions, results draft, graph critique feedback</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Not every graph belongs in the report</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CER organizer, limitations organizer, discussion draft, future work paragraph</x:t>
   </x:si>
   <x:si>
@@ -426,9 +420,6 @@
     <x:t xml:space="preserve">Peer review forms, revision plan, revised Draft 2</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Conversation matters more than the form alone</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Visual aid, speaking notes, practice feedback, presentation reflection</x:t>
   </x:si>
   <x:si>
@@ -520,213 +511,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Teacher Move</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Course launch</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students understand STARLAB culture and research expectations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Collect launch reflection and identity inventory</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Preliminary project pitch</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have at least one promising research direction</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Do not require final project decisions yet</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Formal research plan approval</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Pilot testing launch</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students test a small piece of their method or design</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Require journal setup and safety check</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 6-7</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Method revision gate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Check revised procedures and data tables</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">First data checkpoint</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students show raw data and documentation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 12</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mid-project progress report</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students summarize completed work, preliminary evidence, challenges, and next steps</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Create recovery plans for students with limited data</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 16</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Readiness for analysis</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have organized data and limitations identified</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Approve Unit 4 readiness categories</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 17</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Clean data audit</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Raw data preserved and clean data copy created</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Stop analysis if data are not understandable</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 18</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Analysis plan checkpoint</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students choose calculations/statistics/metrics that fit their question</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Avoid unnecessary advanced methods</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 19</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visual and limitations review</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Graphs/visuals are clear and honest; limitations are named</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Check labels, units, captions, error/uncertainty</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 20</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 5 readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have interpretation notes and analysis summary</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Prevent overclaiming before report writing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 21</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students map project evidence into report sections</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 26</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Complete Draft 1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students submit a complete imperfect report draft</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Make revision possible</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 27</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Peer review and revision</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students complete structured peer review and revision plan</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Require specific, evidence-based feedback</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 28</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students have visual aid and practice presentation feedback</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 31</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Q&amp;A readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students prepare evidence-based responses to likely questions</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Teach scientific humility and limitations language</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Showcase readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Final visual product and logistics are ready</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Confirm backup plans and professionalism expectations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 33</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Week 34</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Portfolio and reflection</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Students complete portfolio, final reflection, and next-step plan</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Collect feedback to improve next STARLAB cycle</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Weekly Print Queue</x:t>
@@ -1273,7 +1057,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table_5" displayName="Table_5" ref="A5:E25">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table_5" displayName="Table_5" ref="A5:E26" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Timing"/>
     <x:tableColumn id="2" name="Checkpoint"/>
@@ -3466,7 +3250,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74314cd53b5741f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12e25d97e8734867"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4127,7 +3911,7 @@
         <x:v>U4 App L; U4 App M; U4 App O; U4 App P; U4 App Q</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="36" hidden="0" customHeight="1">
+    <x:row r="26" ht="58" hidden="0" customHeight="1">
       <x:c r="A26" s="7">
         <x:v>21.0</x:v>
       </x:c>
@@ -4148,10 +3932,10 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H26" s="7" t="str">
-        <x:v>Shift students into scientific structure; set or confirm public showcase format, date, audience, and space six to eight weeks ahead</x:v>
-      </x:c>
-      <x:c r="I26" s="7" t="s">
-        <x:v>121</x:v>
+        <x:v>Teacher-only showcase milestone 1: select the public format, tentative Week 33 date/time, audience, venue, and administrative or district support.</x:v>
+      </x:c>
+      <x:c r="I26" s="7" t="str">
+        <x:v>Planning only; no added student deliverable or print requirement. This is approximately 12 weeks before the required public presentation.</x:v>
       </x:c>
       <x:c r="J26" s="13" t="str">
         <x:v>U5 App R; U5 App S</x:v>
@@ -4175,13 +3959,13 @@
         <x:v>U5 H3; U5 App B; U5 App C</x:v>
       </x:c>
       <x:c r="G27" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="H27" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="H27" s="7" t="s">
+      <x:c r="I27" s="7" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="I27" s="7" t="s">
-        <x:v>124</x:v>
       </x:c>
       <x:c r="J27" s="14"/>
     </x:row>
@@ -4203,17 +3987,17 @@
         <x:v>U5 H4; U5 App D; U5 App E</x:v>
       </x:c>
       <x:c r="G28" s="7" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="H28" s="7" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="H28" s="7" t="s">
+      <x:c r="I28" s="7" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="I28" s="7" t="s">
-        <x:v>127</x:v>
-      </x:c>
       <x:c r="J28" s="13"/>
     </x:row>
-    <x:row r="29" ht="24" hidden="0" customHeight="1">
+    <x:row r="29" ht="58" hidden="0" customHeight="1">
       <x:c r="A29" s="7">
         <x:v>24.0</x:v>
       </x:c>
@@ -4231,13 +4015,13 @@
         <x:v>U5 H5; U5 App F; U5 App G</x:v>
       </x:c>
       <x:c r="G29" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
-        <x:v>Separate results from discussion; send invitations or confirm the public audience and district communication plan</x:v>
-      </x:c>
-      <x:c r="I29" s="7" t="s">
-        <x:v>129</x:v>
+        <x:v>Teacher-only showcase milestone 2: reserve space, confirm the public audience pathway, send a save-the-date, and begin district communication.</x:v>
+      </x:c>
+      <x:c r="I29" s="7" t="str">
+        <x:v>Planning only; no added student deliverable or print requirement. Confirm accessibility, visitor procedures, and communication approvals.</x:v>
       </x:c>
       <x:c r="J29" s="14"/>
     </x:row>
@@ -4259,13 +4043,13 @@
         <x:v>U5 H6; U5 App H; U5 App I</x:v>
       </x:c>
       <x:c r="G30" s="7" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="H30" s="7" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="I30" s="7" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="H30" s="7" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="I30" s="7" t="s">
-        <x:v>132</x:v>
       </x:c>
       <x:c r="J30" s="13"/>
     </x:row>
@@ -4287,17 +4071,17 @@
         <x:v>U5 H7; U5 App J; U5 App K; U5 App L</x:v>
       </x:c>
       <x:c r="G31" s="7" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="H31" s="7" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="I31" s="7" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="H31" s="7" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="I31" s="7" t="s">
-        <x:v>135</x:v>
-      </x:c>
       <x:c r="J31" s="14"/>
     </x:row>
-    <x:row r="32" ht="24" hidden="0" customHeight="1">
+    <x:row r="32" ht="64" hidden="0" customHeight="1">
       <x:c r="A32" s="7">
         <x:v>27.0</x:v>
       </x:c>
@@ -4315,13 +4099,13 @@
         <x:v>U5 H8; U5 H9; U5 App M; U5 App N</x:v>
       </x:c>
       <x:c r="G32" s="7" t="s">
-        <x:v>136</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="H32" s="7" t="str">
-        <x:v>Structure specific peer feedback; finalize public event logistics, technology, accessibility, and assessment workflow</x:v>
-      </x:c>
-      <x:c r="I32" s="7" t="s">
-        <x:v>137</x:v>
+        <x:v>Structure specific peer feedback; teacher-only showcase milestone 3: send formal invitations and lock technology, accessibility, room flow, and assessment workflow.</x:v>
+      </x:c>
+      <x:c r="I32" s="7" t="str">
+        <x:v>No added student deliverable or print requirement; establish logistics owners and backup plans before Unit 6 begins.</x:v>
       </x:c>
       <x:c r="J32" s="13"/>
     </x:row>
@@ -4343,13 +4127,13 @@
         <x:v>U5 H10; U5 H11; U5 App O</x:v>
       </x:c>
       <x:c r="G33" s="7" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="H33" s="7" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="I33" s="7" t="s">
-        <x:v>140</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="J33" s="14" t="str">
         <x:v>U5 App Q; U6 App L</x:v>
@@ -4373,13 +4157,13 @@
         <x:v>U6 H1; U6 H2; U6 H3; U6 App A; U6 App B; U6 App C</x:v>
       </x:c>
       <x:c r="G34" s="7" t="s">
-        <x:v>141</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="H34" s="7" t="s">
-        <x:v>142</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="I34" s="7" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="J34" s="13" t="str">
         <x:v>U6 App L</x:v>
@@ -4403,13 +4187,13 @@
         <x:v>U6 H4; U6 H5; U6 H6; U6 App D; U6 App E</x:v>
       </x:c>
       <x:c r="G35" s="7" t="s">
-        <x:v>144</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="H35" s="7" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="I35" s="7" t="s">
-        <x:v>146</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="J35" s="14" t="str">
         <x:v>U6 App L</x:v>
@@ -4433,13 +4217,13 @@
         <x:v>U6 H7; U6 H8; U6 H9; U6 App F; U6 App G; U6 App H</x:v>
       </x:c>
       <x:c r="G36" s="7" t="s">
-        <x:v>147</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="H36" s="7" t="s">
-        <x:v>148</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="I36" s="7" t="s">
-        <x:v>149</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="J36" s="13" t="str">
         <x:v>U6 App L</x:v>
@@ -4463,13 +4247,13 @@
         <x:v>U6 H10; U6 H11; U6 H12</x:v>
       </x:c>
       <x:c r="G37" s="7" t="s">
-        <x:v>150</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="H37" s="7" t="s">
-        <x:v>151</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="I37" s="7" t="s">
-        <x:v>152</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="J37" s="14" t="str">
         <x:v>U6 App I; U6 App J; U6 App K; U6 App L</x:v>
@@ -4523,13 +4307,13 @@
         <x:v>U6 H15; U6 H16; U6 H18</x:v>
       </x:c>
       <x:c r="G39" s="7" t="s">
-        <x:v>153</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="H39" s="7" t="s">
-        <x:v>154</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="I39" s="7" t="s">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="J39" s="14" t="str">
         <x:v>U6 H17; U6 App O; U6 App P; U6 App Q; U6 App R; U6 App S</x:v>
@@ -5960,7 +5744,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cedb62434d44ae9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57671087f291436a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5983,7 +5767,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" hidden="0" customHeight="1">
       <x:c r="A1" s="17" t="s">
-        <x:v>156</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B1" s="22"/>
       <x:c r="C1" s="22"/>
@@ -8188,7 +7972,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdd4af4819784406"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R107d9862df324966"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8208,12 +7992,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>157</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>158</x:v>
+        <x:v>155</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -8239,16 +8023,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="s">
         <x:v>159</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="F5" s="6" t="s">
-        <x:v>162</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
@@ -10155,7 +9939,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5044cccf93447d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa2727dba07847d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10173,12 +9957,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>163</x:v>
+        <x:v>160</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>164</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -10198,16 +9982,16 @@
     </x:row>
     <x:row r="5" ht="31.5" customHeight="1">
       <x:c r="A5" s="6" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="s">
         <x:v>165</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="s">
-        <x:v>168</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
         <x:v>9</x:v>
@@ -10219,20 +10003,20 @@
       <x:c r="J5" s="4"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="7" t="s">
-        <x:v>169</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="D6" s="7" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="s">
-        <x:v>15</x:v>
+      <x:c r="A6" s="7" t="str">
+        <x:v>Week 1</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="str">
+        <x:v>Course launch</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="str">
+        <x:v>Students understand STARLAB culture and research expectations</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="str">
+        <x:v>Collect launch reflection and identity inventory</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="str">
+        <x:v>Unit 1</x:v>
       </x:c>
       <x:c r="F6" s="4"/>
       <x:c r="G6" s="4"/>
@@ -10241,20 +10025,20 @@
       <x:c r="J6" s="4"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="7" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="D7" s="7" t="s">
-        <x:v>176</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="s">
-        <x:v>15</x:v>
+      <x:c r="A7" s="7" t="str">
+        <x:v>Week 2</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="str">
+        <x:v>Preliminary project pitch</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="str">
+        <x:v>Students have at least one promising research direction</x:v>
+      </x:c>
+      <x:c r="D7" s="7" t="str">
+        <x:v>Do not require final project decisions yet</x:v>
+      </x:c>
+      <x:c r="E7" s="7" t="str">
+        <x:v>Unit 1</x:v>
       </x:c>
       <x:c r="F7" s="4"/>
       <x:c r="G7" s="4"/>
@@ -10263,11 +10047,11 @@
       <x:c r="J7" s="4"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="7" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="s">
-        <x:v>178</x:v>
+      <x:c r="A8" s="7" t="str">
+        <x:v>Week 4</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="str">
+        <x:v>Formal research plan approval</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
         <x:v>Students hold an exact Project Approval Tracker status and have concrete next steps</x:v>
@@ -10275,8 +10059,8 @@
       <x:c r="D8" s="7" t="str">
         <x:v>Use the tracker as the official approval record; no testing without Approved for Pilot Testing</x:v>
       </x:c>
-      <x:c r="E8" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="E8" s="7" t="str">
+        <x:v>Unit 2</x:v>
       </x:c>
       <x:c r="F8" s="4"/>
       <x:c r="G8" s="4"/>
@@ -10285,20 +10069,20 @@
       <x:c r="J8" s="4"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="7" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="s">
-        <x:v>181</x:v>
-      </x:c>
-      <x:c r="D9" s="7" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="E9" s="7" t="s">
-        <x:v>27</x:v>
+      <x:c r="A9" s="7" t="str">
+        <x:v>Week 5</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="str">
+        <x:v>Pilot testing launch</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="str">
+        <x:v>Students test a small piece of their method or design</x:v>
+      </x:c>
+      <x:c r="D9" s="7" t="str">
+        <x:v>Require journal setup and safety check</x:v>
+      </x:c>
+      <x:c r="E9" s="7" t="str">
+        <x:v>Unit 3</x:v>
       </x:c>
       <x:c r="F9" s="4"/>
       <x:c r="G9" s="4"/>
@@ -10307,20 +10091,20 @@
       <x:c r="J9" s="4"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="7" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="B10" s="7" t="s">
-        <x:v>184</x:v>
+      <x:c r="A10" s="7" t="str">
+        <x:v>Week 6-7</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="str">
+        <x:v>Method revision gate</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
         <x:v>Students revise, retest, or receive Approved for Systematic Data Collection in the tracker</x:v>
       </x:c>
-      <x:c r="D10" s="7" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="E10" s="7" t="s">
-        <x:v>27</x:v>
+      <x:c r="D10" s="7" t="str">
+        <x:v>Check revised procedures and data tables</x:v>
+      </x:c>
+      <x:c r="E10" s="7" t="str">
+        <x:v>Unit 3</x:v>
       </x:c>
       <x:c r="F10" s="4"/>
       <x:c r="G10" s="4"/>
@@ -10329,20 +10113,20 @@
       <x:c r="J10" s="4"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>188</x:v>
+      <x:c r="A11" s="7" t="str">
+        <x:v>Week 8</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="str">
+        <x:v>First data checkpoint</x:v>
+      </x:c>
+      <x:c r="C11" s="7" t="str">
+        <x:v>Students show raw data and documentation</x:v>
       </x:c>
       <x:c r="D11" s="7" t="str">
         <x:v>Record Approved for Systematic Data Collection before full collection begins</x:v>
       </x:c>
-      <x:c r="E11" s="7" t="s">
-        <x:v>27</x:v>
+      <x:c r="E11" s="7" t="str">
+        <x:v>Unit 3</x:v>
       </x:c>
       <x:c r="F11" s="4"/>
       <x:c r="G11" s="4"/>
@@ -10351,20 +10135,20 @@
       <x:c r="J11" s="4"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="7" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="B12" s="7" t="s">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="D12" s="7" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="E12" s="7" t="s">
-        <x:v>27</x:v>
+      <x:c r="A12" s="7" t="str">
+        <x:v>Week 12</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="str">
+        <x:v>Mid-project progress report</x:v>
+      </x:c>
+      <x:c r="C12" s="7" t="str">
+        <x:v>Students summarize completed work, preliminary evidence, challenges, and next steps</x:v>
+      </x:c>
+      <x:c r="D12" s="7" t="str">
+        <x:v>Create recovery plans for students with limited data</x:v>
+      </x:c>
+      <x:c r="E12" s="7" t="str">
+        <x:v>Unit 3</x:v>
       </x:c>
       <x:c r="F12" s="4"/>
       <x:c r="G12" s="4"/>
@@ -10373,20 +10157,20 @@
       <x:c r="J12" s="4"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="s">
-        <x:v>193</x:v>
-      </x:c>
-      <x:c r="B13" s="7" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="D13" s="7" t="s">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="s">
-        <x:v>27</x:v>
+      <x:c r="A13" s="7" t="str">
+        <x:v>Week 16</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="str">
+        <x:v>Readiness for analysis</x:v>
+      </x:c>
+      <x:c r="C13" s="7" t="str">
+        <x:v>Students have organized data and limitations identified</x:v>
+      </x:c>
+      <x:c r="D13" s="7" t="str">
+        <x:v>Approve Unit 4 readiness categories</x:v>
+      </x:c>
+      <x:c r="E13" s="7" t="str">
+        <x:v>Unit 3</x:v>
       </x:c>
       <x:c r="F13" s="4"/>
       <x:c r="G13" s="4"/>
@@ -10395,20 +10179,20 @@
       <x:c r="J13" s="4"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="7" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="B14" s="7" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="s">
-        <x:v>199</x:v>
-      </x:c>
-      <x:c r="D14" s="7" t="s">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="s">
-        <x:v>33</x:v>
+      <x:c r="A14" s="7" t="str">
+        <x:v>Week 17</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="str">
+        <x:v>Clean data audit</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="str">
+        <x:v>Raw data preserved and clean data copy created</x:v>
+      </x:c>
+      <x:c r="D14" s="7" t="str">
+        <x:v>Stop analysis if data are not understandable</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="str">
+        <x:v>Unit 4</x:v>
       </x:c>
       <x:c r="F14" s="4"/>
       <x:c r="G14" s="4"/>
@@ -10417,20 +10201,20 @@
       <x:c r="J14" s="4"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="7" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="D15" s="7" t="s">
-        <x:v>204</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="s">
-        <x:v>33</x:v>
+      <x:c r="A15" s="7" t="str">
+        <x:v>Week 18</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="str">
+        <x:v>Analysis plan checkpoint</x:v>
+      </x:c>
+      <x:c r="C15" s="7" t="str">
+        <x:v>Students choose calculations/statistics/metrics that fit their question</x:v>
+      </x:c>
+      <x:c r="D15" s="7" t="str">
+        <x:v>Avoid unnecessary advanced methods</x:v>
+      </x:c>
+      <x:c r="E15" s="7" t="str">
+        <x:v>Unit 4</x:v>
       </x:c>
       <x:c r="F15" s="4"/>
       <x:c r="G15" s="4"/>
@@ -10439,20 +10223,20 @@
       <x:c r="J15" s="4"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="7" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>207</x:v>
-      </x:c>
-      <x:c r="D16" s="7" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="E16" s="7" t="s">
-        <x:v>33</x:v>
+      <x:c r="A16" s="7" t="str">
+        <x:v>Week 19</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="str">
+        <x:v>Visual and limitations review</x:v>
+      </x:c>
+      <x:c r="C16" s="7" t="str">
+        <x:v>Graphs/visuals are clear and honest; limitations are named</x:v>
+      </x:c>
+      <x:c r="D16" s="7" t="str">
+        <x:v>Check labels, units, captions, error/uncertainty</x:v>
+      </x:c>
+      <x:c r="E16" s="7" t="str">
+        <x:v>Unit 4</x:v>
       </x:c>
       <x:c r="F16" s="4"/>
       <x:c r="G16" s="4"/>
@@ -10461,20 +10245,20 @@
       <x:c r="J16" s="4"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="7" t="s">
-        <x:v>209</x:v>
-      </x:c>
-      <x:c r="B17" s="7" t="s">
-        <x:v>210</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="D17" s="7" t="s">
-        <x:v>212</x:v>
-      </x:c>
-      <x:c r="E17" s="7" t="s">
-        <x:v>33</x:v>
+      <x:c r="A17" s="7" t="str">
+        <x:v>Week 20</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="str">
+        <x:v>Unit 5 readiness</x:v>
+      </x:c>
+      <x:c r="C17" s="7" t="str">
+        <x:v>Students have interpretation notes and analysis summary</x:v>
+      </x:c>
+      <x:c r="D17" s="7" t="str">
+        <x:v>Prevent overclaiming before report writing</x:v>
+      </x:c>
+      <x:c r="E17" s="7" t="str">
+        <x:v>Unit 4</x:v>
       </x:c>
       <x:c r="F17" s="4"/>
       <x:c r="G17" s="4"/>
@@ -10482,21 +10266,21 @@
       <x:c r="I17" s="4"/>
       <x:c r="J17" s="4"/>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="7" t="s">
-        <x:v>213</x:v>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="7" t="str">
+        <x:v>Week 21</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>Report and public showcase planning launch</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="s">
-        <x:v>214</x:v>
+        <x:v>Showcase milestone 1: event framework</x:v>
+      </x:c>
+      <x:c r="C18" s="7" t="str">
+        <x:v>No additional student product; regular report planning continues.</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
-        <x:v>Set public format, target date, audience, and space six to eight weeks ahead</x:v>
-      </x:c>
-      <x:c r="E18" s="7" t="s">
-        <x:v>39</x:v>
+        <x:v>Select the public format, tentative Week 33 date/time, audience, venue, and administrative or district support.</x:v>
+      </x:c>
+      <x:c r="E18" s="7" t="str">
+        <x:v>Unit 5</x:v>
       </x:c>
       <x:c r="F18" s="4"/>
       <x:c r="G18" s="4"/>
@@ -10504,21 +10288,21 @@
       <x:c r="I18" s="4"/>
       <x:c r="J18" s="4"/>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="7" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B19" s="7" t="s">
-        <x:v>216</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>217</x:v>
-      </x:c>
-      <x:c r="D19" s="7" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="E19" s="7" t="s">
-        <x:v>39</x:v>
+    <x:row r="19" ht="48" customHeight="1">
+      <x:c r="A19" s="7" t="str">
+        <x:v>Week 24</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="str">
+        <x:v>Showcase milestone 2: audience and space confirmation</x:v>
+      </x:c>
+      <x:c r="C19" s="7" t="str">
+        <x:v>No additional student product; regular results work continues.</x:v>
+      </x:c>
+      <x:c r="D19" s="7" t="str">
+        <x:v>Reserve space, confirm the public audience pathway, send a save-the-date, and begin district communication.</x:v>
+      </x:c>
+      <x:c r="E19" s="7" t="str">
+        <x:v>Unit 5</x:v>
       </x:c>
       <x:c r="F19" s="4"/>
       <x:c r="G19" s="4"/>
@@ -10527,20 +10311,20 @@
       <x:c r="J19" s="4"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="7" t="s">
-        <x:v>219</x:v>
-      </x:c>
-      <x:c r="B20" s="7" t="s">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="D20" s="7" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="E20" s="7" t="s">
-        <x:v>39</x:v>
+      <x:c r="A20" s="7" t="str">
+        <x:v>Week 26</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="str">
+        <x:v>Complete Draft 1</x:v>
+      </x:c>
+      <x:c r="C20" s="7" t="str">
+        <x:v>Students submit a complete imperfect report draft</x:v>
+      </x:c>
+      <x:c r="D20" s="7" t="str">
+        <x:v>Make revision possible</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="str">
+        <x:v>Unit 5</x:v>
       </x:c>
       <x:c r="F20" s="4"/>
       <x:c r="G20" s="4"/>
@@ -10548,21 +10332,21 @@
       <x:c r="I20" s="4"/>
       <x:c r="J20" s="4"/>
     </x:row>
-    <x:row r="21" ht="15.75" customHeight="1">
-      <x:c r="A21" s="7" t="s">
-        <x:v>223</x:v>
+    <x:row r="21" ht="48" customHeight="1">
+      <x:c r="A21" s="7" t="str">
+        <x:v>Week 27</x:v>
       </x:c>
       <x:c r="B21" s="7" t="str">
-        <x:v>Presentation product and event readiness</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="s">
-        <x:v>224</x:v>
+        <x:v>Peer review plus showcase milestone 3</x:v>
+      </x:c>
+      <x:c r="C21" s="7" t="str">
+        <x:v>Students complete structured peer review and a revision plan; no additional showcase deliverable.</x:v>
       </x:c>
       <x:c r="D21" s="7" t="str">
-        <x:v>Check readability and presentation story; finalize public event logistics</x:v>
-      </x:c>
-      <x:c r="E21" s="7" t="s">
-        <x:v>39</x:v>
+        <x:v>Require evidence-based feedback; send formal invitations and lock technology, accessibility, room flow, and assessment workflow.</x:v>
+      </x:c>
+      <x:c r="E21" s="7" t="str">
+        <x:v>Unit 5</x:v>
       </x:c>
       <x:c r="F21" s="4"/>
       <x:c r="G21" s="4"/>
@@ -10571,20 +10355,20 @@
       <x:c r="J21" s="4"/>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
-      <x:c r="A22" s="7" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="B22" s="7" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="D22" s="7" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="E22" s="7" t="s">
-        <x:v>45</x:v>
+      <x:c r="A22" s="7" t="str">
+        <x:v>Week 28</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="str">
+        <x:v>Presentation product and event readiness</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="str">
+        <x:v>Students have visual aid and practice presentation feedback</x:v>
+      </x:c>
+      <x:c r="D22" s="7" t="str">
+        <x:v>Check readability and presentation story; finalize public event logistics</x:v>
+      </x:c>
+      <x:c r="E22" s="7" t="str">
+        <x:v>Unit 5</x:v>
       </x:c>
       <x:c r="F22" s="4"/>
       <x:c r="G22" s="4"/>
@@ -10593,20 +10377,20 @@
       <x:c r="J22" s="4"/>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
-      <x:c r="A23" s="7" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="B23" s="7" t="s">
-        <x:v>230</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="D23" s="7" t="s">
-        <x:v>232</x:v>
-      </x:c>
-      <x:c r="E23" s="7" t="s">
-        <x:v>45</x:v>
+      <x:c r="A23" s="7" t="str">
+        <x:v>Week 31</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="str">
+        <x:v>Q&amp;A readiness</x:v>
+      </x:c>
+      <x:c r="C23" s="7" t="str">
+        <x:v>Students prepare evidence-based responses to likely questions</x:v>
+      </x:c>
+      <x:c r="D23" s="7" t="str">
+        <x:v>Teach scientific humility and limitations language</x:v>
+      </x:c>
+      <x:c r="E23" s="7" t="str">
+        <x:v>Unit 6</x:v>
       </x:c>
       <x:c r="F23" s="4"/>
       <x:c r="G23" s="4"/>
@@ -10615,20 +10399,20 @@
       <x:c r="J23" s="4"/>
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
-      <x:c r="A24" s="7" t="s">
-        <x:v>233</x:v>
+      <x:c r="A24" s="7" t="str">
+        <x:v>Week 32</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
-        <x:v>Required public presentation/showcase</x:v>
+        <x:v>Showcase readiness</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
-        <x:v>Students present their research to a genuine public audience</x:v>
+        <x:v>Final visual product and logistics are ready</x:v>
       </x:c>
       <x:c r="D24" s="7" t="str">
-        <x:v>Collect audience feedback and score with Unit 6 Appendices L and M</x:v>
-      </x:c>
-      <x:c r="E24" s="7" t="s">
-        <x:v>45</x:v>
+        <x:v>Confirm backup plans and professionalism expectations</x:v>
+      </x:c>
+      <x:c r="E24" s="7" t="str">
+        <x:v>Unit 6</x:v>
       </x:c>
       <x:c r="F24" s="4"/>
       <x:c r="G24" s="4"/>
@@ -10637,20 +10421,20 @@
       <x:c r="J24" s="4"/>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
-      <x:c r="A25" s="7" t="s">
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="B25" s="7" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="C25" s="7" t="s">
-        <x:v>236</x:v>
-      </x:c>
-      <x:c r="D25" s="7" t="s">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="E25" s="7" t="s">
-        <x:v>45</x:v>
+      <x:c r="A25" s="7" t="str">
+        <x:v>Week 33</x:v>
+      </x:c>
+      <x:c r="B25" s="7" t="str">
+        <x:v>Required public presentation/showcase</x:v>
+      </x:c>
+      <x:c r="C25" s="7" t="str">
+        <x:v>Students present their research to a genuine public audience</x:v>
+      </x:c>
+      <x:c r="D25" s="7" t="str">
+        <x:v>Collect audience feedback and score with Unit 6 Appendices L and M</x:v>
+      </x:c>
+      <x:c r="E25" s="7" t="str">
+        <x:v>Unit 6</x:v>
       </x:c>
       <x:c r="F25" s="4"/>
       <x:c r="G25" s="4"/>
@@ -10659,11 +10443,21 @@
       <x:c r="J25" s="4"/>
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1">
-      <x:c r="A26" s="4"/>
-      <x:c r="B26" s="4"/>
-      <x:c r="C26" s="4"/>
-      <x:c r="D26" s="4"/>
-      <x:c r="E26" s="4"/>
+      <x:c r="A26" s="4" t="str">
+        <x:v>Week 34</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="str">
+        <x:v>Portfolio and reflection</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>Students complete portfolio, final reflection, and next-step plan</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>Collect feedback to improve next STARLAB cycle</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="str">
+        <x:v>Unit 6</x:v>
+      </x:c>
       <x:c r="F26" s="4"/>
       <x:c r="G26" s="4"/>
       <x:c r="H26" s="4"/>
@@ -12246,7 +12040,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae3c4313a7248c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8810027aac0747dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12266,12 +12060,12 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>238</x:v>
+        <x:v>166</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>239</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
@@ -12300,13 +12094,13 @@
         <x:v>Deck Use</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
-        <x:v>240</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="E5" s="6" t="s">
-        <x:v>241</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="F5" s="6" t="s">
-        <x:v>242</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
@@ -12816,7 +12610,7 @@
       </x:c>
       <x:c r="E27" s="7"/>
       <x:c r="F27" s="7" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="G27" s="4"/>
       <x:c r="H27" s="4"/>
@@ -12838,7 +12632,7 @@
       </x:c>
       <x:c r="E28" s="7"/>
       <x:c r="F28" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="G28" s="4"/>
       <x:c r="H28" s="4"/>
@@ -12860,7 +12654,7 @@
       </x:c>
       <x:c r="E29" s="7"/>
       <x:c r="F29" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="G29" s="4"/>
       <x:c r="H29" s="4"/>
@@ -12882,7 +12676,7 @@
       </x:c>
       <x:c r="E30" s="7"/>
       <x:c r="F30" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="G30" s="4"/>
       <x:c r="H30" s="4"/>
@@ -12904,7 +12698,7 @@
       </x:c>
       <x:c r="E31" s="7"/>
       <x:c r="F31" s="7" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="G31" s="4"/>
       <x:c r="H31" s="4"/>
@@ -12926,7 +12720,7 @@
       </x:c>
       <x:c r="E32" s="7"/>
       <x:c r="F32" s="7" t="s">
-        <x:v>136</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="G32" s="4"/>
       <x:c r="H32" s="4"/>
@@ -12950,7 +12744,7 @@
         <x:v>U5 App Q; U6 App L</x:v>
       </x:c>
       <x:c r="F33" s="7" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="G33" s="4"/>
       <x:c r="H33" s="4"/>
@@ -12974,7 +12768,7 @@
         <x:v>U6 App L</x:v>
       </x:c>
       <x:c r="F34" s="7" t="s">
-        <x:v>141</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="G34" s="4"/>
       <x:c r="H34" s="4"/>
@@ -12998,7 +12792,7 @@
         <x:v>U6 App L</x:v>
       </x:c>
       <x:c r="F35" s="7" t="s">
-        <x:v>144</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="G35" s="4"/>
       <x:c r="H35" s="4"/>
@@ -13022,7 +12816,7 @@
         <x:v>U6 App L</x:v>
       </x:c>
       <x:c r="F36" s="7" t="s">
-        <x:v>147</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="G36" s="4"/>
       <x:c r="H36" s="4"/>
@@ -13046,7 +12840,7 @@
         <x:v>U6 App I; U6 App J; U6 App K; U6 App L</x:v>
       </x:c>
       <x:c r="F37" s="7" t="s">
-        <x:v>150</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="G37" s="4"/>
       <x:c r="H37" s="4"/>
@@ -13070,7 +12864,7 @@
         <x:v>U6 App N</x:v>
       </x:c>
       <x:c r="F38" s="7" t="s">
-        <x:v>243</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="G38" s="4"/>
       <x:c r="H38" s="4"/>
@@ -13094,7 +12888,7 @@
         <x:v>U6 H17; U6 App O; U6 App P; U6 App Q; U6 App R; U6 App S</x:v>
       </x:c>
       <x:c r="F39" s="7" t="s">
-        <x:v>153</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="G39" s="4"/>
       <x:c r="H39" s="4"/>
@@ -14521,7 +14315,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8209c34c3df467d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a8329b977b346fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish authoritative assessment tools
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
+++ b/Teacher Resources (Start Here)/05_STARLAB_Full_Course_Implementation_Calendar.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R33580968ffa4498f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="R004d08fdd2d84867"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="R37485dac14564475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R06669ac9983f4136"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="Rda452686af514614"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="R01fd915949cc4b57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rdc134e59d49e4fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34-Week Calendar" sheetId="2" r:id="R2849f4339ea2471c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck Alignment" sheetId="3" r:id="R01350a8f669d4327"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Overview" sheetId="4" r:id="R222e1370355d4c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Major Checkpoints" sheetId="5" r:id="Rcb0843496b014cab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Queue" sheetId="6" r:id="R2d9d4abf685a4567"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3250,7 +3250,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12e25d97e8734867"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf614fe5f74744829"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3473,7 +3473,9 @@
       <x:c r="I10" s="7" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="J10" s="13"/>
+      <x:c r="J10" s="13" t="str">
+        <x:v>U3 App V</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="7">
@@ -3678,7 +3680,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="J17" s="14" t="str">
-        <x:v>U3 App O</x:v>
+        <x:v>U3 App O; U3 App V</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" hidden="0" customHeight="1">
@@ -3794,7 +3796,7 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="J21" s="14" t="str">
-        <x:v>U3 App S; U3 App T; U3 App U</x:v>
+        <x:v>U3 App S; U3 App T; U3 App U; U3 App V</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
@@ -4107,7 +4109,9 @@
       <x:c r="I32" s="7" t="str">
         <x:v>No added student deliverable or print requirement; establish logistics owners and backup plans before Unit 6 begins.</x:v>
       </x:c>
-      <x:c r="J32" s="13"/>
+      <x:c r="J32" s="13" t="str">
+        <x:v>U5 App T</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="7">
@@ -5744,7 +5748,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57671087f291436a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc1e69ab63d24df2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6022,7 +6026,9 @@
       <x:c r="F12" s="53" t="str">
         <x:v>Week 5: U3 H1-H3; U3 Apps A-C</x:v>
       </x:c>
-      <x:c r="G12" s="54" t="str"/>
+      <x:c r="G12" s="54" t="str">
+        <x:v>Week 5 and ongoing: U3 App V</x:v>
+      </x:c>
       <x:c r="H12" s="64" t="str">
         <x:v>Journal setup and scientific documentation</x:v>
       </x:c>
@@ -6247,7 +6253,8 @@
         <x:v>Week 27: U5 H8-H9; U5 Apps M-N</x:v>
       </x:c>
       <x:c r="G20" s="54" t="str">
-        <x:v>Previously issued reference: U5 Apps J-L</x:v>
+        <x:v>Previously issued reference: U5 Apps J-L
+Week 27 optional scoring reference: U5 App T</x:v>
       </x:c>
       <x:c r="H20" s="64" t="str">
         <x:v>Structured feedback and revision</x:v>
@@ -7972,7 +7979,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R107d9862df324966"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1353e11404364cbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9939,7 +9946,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa2727dba07847d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d03509323f0409d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12040,7 +12047,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8810027aac0747dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c346f724e24687"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12216,7 +12223,9 @@
       <x:c r="D10" s="7" t="str">
         <x:v>U3 H1; U3 H2; U3 H3; U3 App A; U3 App B; U3 App C</x:v>
       </x:c>
-      <x:c r="E10" s="7"/>
+      <x:c r="E10" s="7" t="str">
+        <x:v>U3 App V</x:v>
+      </x:c>
       <x:c r="F10" s="7" t="s">
         <x:v>72</x:v>
       </x:c>
@@ -12379,7 +12388,7 @@
         <x:v>U3 H14; U3 App N</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
-        <x:v>U3 App O</x:v>
+        <x:v>U3 App O; U3 App V</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
         <x:v>93</x:v>
@@ -12471,7 +12480,7 @@
         <x:v>U3 H18; U3 H19</x:v>
       </x:c>
       <x:c r="E21" s="7" t="str">
-        <x:v>U3 App S; U3 App T; U3 App U</x:v>
+        <x:v>U3 App S; U3 App T; U3 App U; U3 App V</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
         <x:v>105</x:v>
@@ -12718,7 +12727,9 @@
       <x:c r="D32" s="7" t="str">
         <x:v>U5 H8; U5 H9; U5 App M; U5 App N</x:v>
       </x:c>
-      <x:c r="E32" s="7"/>
+      <x:c r="E32" s="7" t="str">
+        <x:v>U5 App T</x:v>
+      </x:c>
       <x:c r="F32" s="7" t="s">
         <x:v>134</x:v>
       </x:c>
@@ -14315,7 +14326,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a8329b977b346fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5d7448dbcdb4a60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>